<commit_message>
📄 Replace ledger with Chuck's 10:02 upload: 83 open pairs (3 closed→TRADE, +1 new 09-24 1211/6680, 52 stored P/L recalculated, 09-23 pair now buy 9888/sell 9880 @-590)
</commit_message>
<xml_diff>
--- a/data/Record_Sept-24.xlsx
+++ b/data/Record_Sept-24.xlsx
@@ -872,11 +872,11 @@
         <v>25566.0</v>
       </c>
       <c r="C3" s="7">
-        <v>24800.0</v>
+        <v>24695.0</v>
       </c>
       <c r="D3" s="5" t="str">
         <f>(C3-B3)/B3</f>
-        <v>-3.00%</v>
+        <v>-3.41%</v>
       </c>
       <c r="H3" s="5"/>
       <c r="Z3" s="6"/>
@@ -905,7 +905,7 @@
       </c>
       <c r="H5" s="5" t="str">
         <f t="shared" ref="H5:H6" si="1">(I5-K5)/K5-$D$3</f>
-        <v>-4.19%</v>
+        <v>-3.78%</v>
       </c>
       <c r="I5" s="9">
         <v>1.55</v>
@@ -926,7 +926,7 @@
       </c>
       <c r="H6" s="5" t="str">
         <f t="shared" si="1"/>
-        <v>-1.94%</v>
+        <v>-1.53%</v>
       </c>
       <c r="I6" s="11">
         <v>4.24</v>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="H15" s="5" t="str">
         <f t="shared" ref="H15:H16" si="2">(I15-K15)/K15-$D$3</f>
-        <v>-1.47%</v>
+        <v>-1.06%</v>
       </c>
       <c r="I15" s="9">
         <v>38.5</v>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="H16" s="5" t="str">
         <f t="shared" si="2"/>
-        <v>-2.34%</v>
+        <v>-1.93%</v>
       </c>
       <c r="I16" s="11">
         <v>18.11</v>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="H25" s="5" t="str">
         <f t="shared" ref="H25:H26" si="3">(I25-K25)/K25-$D$3</f>
-        <v>-3.45%</v>
+        <v>-3.04%</v>
       </c>
       <c r="I25" s="9">
         <v>90.0</v>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="H26" s="5" t="str">
         <f t="shared" si="3"/>
-        <v>-3.13%</v>
+        <v>-2.72%</v>
       </c>
       <c r="I26" s="11">
         <v>107.2</v>
@@ -1489,10 +1489,10 @@
       </c>
       <c r="H40" s="5" t="str">
         <f t="shared" ref="H40:H41" si="4">(I40-K40)/K40-$D$3</f>
-        <v>-6.98%</v>
+        <v>-10.78%</v>
       </c>
       <c r="I40" s="9">
-        <v>2.03</v>
+        <v>1.935</v>
       </c>
       <c r="J40" s="10">
         <v>968.0</v>
@@ -1510,10 +1510,10 @@
       </c>
       <c r="H41" s="5" t="str">
         <f t="shared" si="4"/>
-        <v>10.85%</v>
+        <v>8.41%</v>
       </c>
       <c r="I41" s="11">
-        <v>0.755</v>
+        <v>0.735</v>
       </c>
       <c r="J41" s="12">
         <v>3800.0</v>
@@ -1536,11 +1536,11 @@
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="15" t="str">
         <f>I41</f>
-        <v> $ 0.76 </v>
+        <v> $ 0.74 </v>
       </c>
       <c r="B43" s="15" t="str">
         <f>I40</f>
-        <v> $ 2.03 </v>
+        <v> $ 1.94 </v>
       </c>
       <c r="C43">
         <v>4000.0</v>
@@ -1603,11 +1603,11 @@
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="14" t="str">
         <f>$B$43</f>
-        <v> $ 2.03 </v>
+        <v> $ 1.94 </v>
       </c>
       <c r="B48" s="14" t="str">
         <f>$A$43</f>
-        <v> $ 0.76 </v>
+        <v> $ 0.74 </v>
       </c>
       <c r="C48">
         <v>12000.0</v>
@@ -1620,11 +1620,11 @@
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="4" t="str">
         <f>(A48-A47)*C49</f>
-        <v>0</v>
+        <v>-380</v>
       </c>
       <c r="B49" s="14" t="str">
         <f>C48*(B47-B48)</f>
-        <v> $ -   </v>
+        <v> $ 240.00 </v>
       </c>
       <c r="C49">
         <v>4000.0</v>
@@ -1634,11 +1634,11 @@
       </c>
       <c r="E49" s="14" t="str">
         <f>A49</f>
-        <v> $ -   </v>
+        <v>-$ 380.00 </v>
       </c>
       <c r="F49" s="14" t="str">
         <f>(B49+A49)</f>
-        <v> $ -   </v>
+        <v>-$ 140.00 </v>
       </c>
       <c r="G49" t="str">
         <f>IF(F49&gt;0, "TRADE","H")</f>
@@ -1676,11 +1676,11 @@
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="14" t="str">
         <f>$B$43</f>
-        <v> $ 2.03 </v>
+        <v> $ 1.94 </v>
       </c>
       <c r="B53" s="14" t="str">
         <f>$A$43</f>
-        <v> $ 0.76 </v>
+        <v> $ 0.74 </v>
       </c>
       <c r="C53">
         <v>12000.0</v>
@@ -1693,11 +1693,11 @@
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="4" t="str">
         <f>(A53-A52)*C54</f>
-        <v>-1300</v>
+        <v>-1680</v>
       </c>
       <c r="B54" s="14" t="str">
         <f>C53*(B52-B53)</f>
-        <v>-$ 60.00 </v>
+        <v> $ 180.00 </v>
       </c>
       <c r="C54">
         <v>4000.0</v>
@@ -1707,11 +1707,11 @@
       </c>
       <c r="E54" s="14" t="str">
         <f>A54</f>
-        <v>-$ 1,300.00 </v>
+        <v>-$ 1,680.00 </v>
       </c>
       <c r="F54" s="14" t="str">
         <f>(B54+A54)</f>
-        <v>-$ 1,360.00 </v>
+        <v>-$ 1,500.00 </v>
       </c>
       <c r="G54" t="str">
         <f>IF(F54&gt;0, "TRADE","H")</f>
@@ -1750,11 +1750,11 @@
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="14" t="str">
         <f>$B$43</f>
-        <v> $ 2.03 </v>
+        <v> $ 1.94 </v>
       </c>
       <c r="B58" s="14" t="str">
         <f>$A$43</f>
-        <v> $ 0.76 </v>
+        <v> $ 0.74 </v>
       </c>
       <c r="C58">
         <v>12000.0</v>
@@ -1767,11 +1767,11 @@
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="4" t="str">
         <f>(A58-A57)*C59</f>
-        <v>-1150.8</v>
+        <v>-1530.8</v>
       </c>
       <c r="B59" s="14" t="str">
         <f>C58*(B57-B58)</f>
-        <v>-$ 840.00 </v>
+        <v>-$ 600.00 </v>
       </c>
       <c r="C59">
         <v>4000.0</v>
@@ -1781,11 +1781,11 @@
       </c>
       <c r="E59" s="14" t="str">
         <f>A59</f>
-        <v>-$ 1,150.80 </v>
+        <v>-$ 1,530.80 </v>
       </c>
       <c r="F59" s="14" t="str">
         <f>(B59+A59)</f>
-        <v>-$ 1,990.80 </v>
+        <v>-$ 2,130.80 </v>
       </c>
       <c r="G59" t="str">
         <f>IF(F59&gt;0, "TRADE","H")</f>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="H60" s="5" t="str">
         <f t="shared" ref="H60:H61" si="5">(I60-K60)/K60-$D$3</f>
-        <v>11.62%</v>
+        <v>12.03%</v>
       </c>
       <c r="I60" s="9">
         <v>0.315</v>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="H61" s="5" t="str">
         <f t="shared" si="5"/>
-        <v>14.45%</v>
+        <v>14.87%</v>
       </c>
       <c r="I61" s="11">
         <v>0.535</v>
@@ -1977,10 +1977,10 @@
       </c>
       <c r="H70" s="5" t="str">
         <f t="shared" ref="H70:H71" si="6">(I70-K70)/K70-$D$3</f>
-        <v>-1.89%</v>
+        <v>-1.98%</v>
       </c>
       <c r="I70" s="9">
-        <v>22.6</v>
+        <v>22.48</v>
       </c>
       <c r="J70" s="10">
         <v>763.0</v>
@@ -1998,10 +1998,10 @@
       </c>
       <c r="H71" s="5" t="str">
         <f t="shared" si="6"/>
-        <v>-6.01%</v>
+        <v>-5.03%</v>
       </c>
       <c r="I71" s="11">
-        <v>64.7</v>
+        <v>65.1</v>
       </c>
       <c r="J71" s="12">
         <v>2382.0</v>
@@ -2020,17 +2020,17 @@
       </c>
       <c r="H72" s="5" t="str">
         <f>H70-H71</f>
-        <v>4.12%</v>
+        <v>3.05%</v>
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="15" t="str">
         <f>I70</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B73" s="15" t="str">
         <f>I71</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C73">
         <v>600.0</v>
@@ -2094,11 +2094,11 @@
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="B78" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="C78" s="16">
         <v>300.0</v>
@@ -2111,11 +2111,11 @@
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="4" t="str">
         <f>(A78-A77)*C78</f>
-        <v>-3720</v>
+        <v>-3600</v>
       </c>
       <c r="B79" s="14" t="str">
         <f>C79*(B77-B78)</f>
-        <v> $ 1,960.00 </v>
+        <v> $ 2,080.00 </v>
       </c>
       <c r="C79" s="16">
         <v>1000.0</v>
@@ -2125,11 +2125,11 @@
       </c>
       <c r="E79" s="14" t="str">
         <f>A79</f>
-        <v>-$ 3,720.00 </v>
+        <v>-$ 3,600.00 </v>
       </c>
       <c r="F79" s="14" t="str">
         <f>(B79+A79)</f>
-        <v>-$ 1,760.00 </v>
+        <v>-$ 1,520.00 </v>
       </c>
       <c r="G79" t="str">
         <f>IF(F79&gt;0, "TRADE","H")</f>
@@ -2169,11 +2169,11 @@
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="B83" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="C83">
         <v>200.0</v>
@@ -2186,11 +2186,11 @@
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="4" t="str">
         <f>(A83-A82)*C83</f>
-        <v>-2260</v>
+        <v>-2180</v>
       </c>
       <c r="B84" s="14" t="str">
         <f>C84*(B82-B83)</f>
-        <v> $ 1,236.00 </v>
+        <v> $ 1,308.00 </v>
       </c>
       <c r="C84">
         <v>600.0</v>
@@ -2200,11 +2200,11 @@
       </c>
       <c r="E84" s="14" t="str">
         <f>A84</f>
-        <v>-$ 2,260.00 </v>
+        <v>-$ 2,180.00 </v>
       </c>
       <c r="F84" s="14" t="str">
         <f>(B84+A84)</f>
-        <v>-$ 1,024.00 </v>
+        <v>-$ 872.00 </v>
       </c>
       <c r="G84" t="str">
         <f>IF(F84&gt;0, "TRADE","H")</f>
@@ -2244,11 +2244,11 @@
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="B88" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="C88">
         <v>200.0</v>
@@ -2261,11 +2261,11 @@
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="4" t="str">
         <f>(A88-A87)*C88</f>
-        <v>-590</v>
+        <v>-510</v>
       </c>
       <c r="B89" s="14" t="str">
         <f>C89*(B87-B88)</f>
-        <v> $ 108.00 </v>
+        <v> $ 180.00 </v>
       </c>
       <c r="C89">
         <v>600.0</v>
@@ -2275,11 +2275,11 @@
       </c>
       <c r="E89" s="14" t="str">
         <f>A89</f>
-        <v>-$ 590.00 </v>
+        <v>-$ 510.00 </v>
       </c>
       <c r="F89" s="14" t="str">
         <f>(B89+A89)</f>
-        <v>-$ 482.00 </v>
+        <v>-$ 330.00 </v>
       </c>
       <c r="G89" t="str">
         <f>IF(F89&gt;0, "TRADE","H")</f>
@@ -2319,11 +2319,11 @@
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="B93" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="C93">
         <v>200.0</v>
@@ -2336,11 +2336,11 @@
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="4" t="str">
         <f>(A93-A92)*C93</f>
-        <v>-480</v>
+        <v>-400</v>
       </c>
       <c r="B94" s="14" t="str">
         <f>C94*(B92-B93)</f>
-        <v> $ 192.00 </v>
+        <v> $ 264.00 </v>
       </c>
       <c r="C94">
         <v>600.0</v>
@@ -2350,11 +2350,11 @@
       </c>
       <c r="E94" s="14" t="str">
         <f>A94</f>
-        <v>-$ 480.00 </v>
+        <v>-$ 400.00 </v>
       </c>
       <c r="F94" s="14" t="str">
         <f>(B94+A94)</f>
-        <v>-$ 288.00 </v>
+        <v>-$ 136.00 </v>
       </c>
       <c r="G94" t="str">
         <f>IF(F94&gt;0, "TRADE","H")</f>
@@ -2394,11 +2394,11 @@
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="B98" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="C98">
         <v>200.0</v>
@@ -2411,11 +2411,11 @@
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="4" t="str">
         <f>(A98-A97)*C98</f>
-        <v>-240</v>
+        <v>-160</v>
       </c>
       <c r="B99" s="14" t="str">
         <f>C99*(B97-B98)</f>
-        <v> $ 204.00 </v>
+        <v> $ 276.00 </v>
       </c>
       <c r="C99">
         <v>600.0</v>
@@ -2425,15 +2425,15 @@
       </c>
       <c r="E99" s="14" t="str">
         <f>A99</f>
-        <v>-$ 240.00 </v>
+        <v>-$ 160.00 </v>
       </c>
       <c r="F99" s="14" t="str">
         <f>(B99+A99)</f>
-        <v>-$ 36.00 </v>
+        <v> $ 116.00 </v>
       </c>
       <c r="G99" t="str">
         <f>IF(F99&gt;0, "TRADE","H")</f>
-        <v>H</v>
+        <v>TRADE</v>
       </c>
       <c r="V99" s="6"/>
     </row>
@@ -2468,11 +2468,11 @@
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B103" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C103">
         <v>600.0</v>
@@ -2485,11 +2485,11 @@
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="4" t="str">
         <f>(A103-A102)*C103</f>
-        <v>-696</v>
+        <v>-768</v>
       </c>
       <c r="B104" s="14" t="str">
         <f>C104*(B102-B103)</f>
-        <v> $ 250.00 </v>
+        <v> $ 170.00 </v>
       </c>
       <c r="C104">
         <v>200.0</v>
@@ -2499,11 +2499,11 @@
       </c>
       <c r="E104" s="14" t="str">
         <f>A104</f>
-        <v>-$ 696.00 </v>
+        <v>-$ 768.00 </v>
       </c>
       <c r="F104" s="14" t="str">
         <f>(B104+A104)</f>
-        <v>-$ 446.00 </v>
+        <v>-$ 598.00 </v>
       </c>
       <c r="G104" t="str">
         <f>IF(F104&gt;0, "TRADE","H")</f>
@@ -2542,11 +2542,11 @@
     <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B108" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C108">
         <v>600.0</v>
@@ -2559,11 +2559,11 @@
     <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="4" t="str">
         <f>(A108-A107)*C108</f>
-        <v>-432</v>
+        <v>-504</v>
       </c>
       <c r="B109" s="14" t="str">
         <f>C109*(B107-B108)</f>
-        <v>-$ 810.00 </v>
+        <v>-$ 890.00 </v>
       </c>
       <c r="C109">
         <v>200.0</v>
@@ -2573,11 +2573,11 @@
       </c>
       <c r="E109" s="14" t="str">
         <f>A109</f>
-        <v>-$ 432.00 </v>
+        <v>-$ 504.00 </v>
       </c>
       <c r="F109" s="14" t="str">
         <f>(B109+A109)</f>
-        <v>-$ 1,242.00 </v>
+        <v>-$ 1,394.00 </v>
       </c>
       <c r="G109" t="str">
         <f>IF(F109&gt;0, "TRADE","H")</f>
@@ -2616,11 +2616,11 @@
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B113" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C113">
         <v>600.0</v>
@@ -2633,11 +2633,11 @@
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="4" t="str">
         <f>(A113-A112)*C113</f>
-        <v>-780</v>
+        <v>-852</v>
       </c>
       <c r="B114" s="14" t="str">
         <f>C114*(B112-B113)</f>
-        <v>-$ 990.00 </v>
+        <v>-$ 1,070.00 </v>
       </c>
       <c r="C114">
         <v>200.0</v>
@@ -2647,11 +2647,11 @@
       </c>
       <c r="E114" s="14" t="str">
         <f>A114</f>
-        <v>-$ 780.00 </v>
+        <v>-$ 852.00 </v>
       </c>
       <c r="F114" s="14" t="str">
         <f>(B114+A114)</f>
-        <v>-$ 1,770.00 </v>
+        <v>-$ 1,922.00 </v>
       </c>
       <c r="G114" t="str">
         <f>IF(F114&gt;0, "TRADE","H")</f>
@@ -2690,11 +2690,11 @@
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B118" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C118">
         <v>600.0</v>
@@ -2707,11 +2707,11 @@
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="4" t="str">
         <f>(A118-A117)*C118</f>
-        <v>-1752</v>
+        <v>-1824</v>
       </c>
       <c r="B119" s="14" t="str">
         <f>C119*(B117-B118)</f>
-        <v>-$ 480.00 </v>
+        <v>-$ 560.00 </v>
       </c>
       <c r="C119">
         <v>200.0</v>
@@ -2721,11 +2721,11 @@
       </c>
       <c r="E119" s="14" t="str">
         <f>A119</f>
-        <v>-$ 1,752.00 </v>
+        <v>-$ 1,824.00 </v>
       </c>
       <c r="F119" s="14" t="str">
         <f>(B119+A119)</f>
-        <v>-$ 2,232.00 </v>
+        <v>-$ 2,384.00 </v>
       </c>
       <c r="G119" t="str">
         <f>IF(F119&gt;0, "TRADE","H")</f>
@@ -2764,11 +2764,11 @@
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B123" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C123">
         <v>600.0</v>
@@ -2781,11 +2781,11 @@
     <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="4" t="str">
         <f>(A123-A122)*C123</f>
-        <v>-1716</v>
+        <v>-1788</v>
       </c>
       <c r="B124" s="14" t="str">
         <f>C124*(B122-B123)</f>
-        <v>-$ 810.00 </v>
+        <v>-$ 890.00 </v>
       </c>
       <c r="C124">
         <v>200.0</v>
@@ -2795,11 +2795,11 @@
       </c>
       <c r="E124" s="14" t="str">
         <f>A124</f>
-        <v>-$ 1,716.00 </v>
+        <v>-$ 1,788.00 </v>
       </c>
       <c r="F124" s="14" t="str">
         <f>(B124+A124)</f>
-        <v>-$ 2,526.00 </v>
+        <v>-$ 2,678.00 </v>
       </c>
       <c r="G124" t="str">
         <f>IF(F124&gt;0, "TRADE","H")</f>
@@ -2838,11 +2838,11 @@
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B128" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C128">
         <v>600.0</v>
@@ -2855,11 +2855,11 @@
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="4" t="str">
         <f>(A128-A127)*C128</f>
-        <v>-1764</v>
+        <v>-1836</v>
       </c>
       <c r="B129" s="14" t="str">
         <f>C129*(B127-B128)</f>
-        <v>-$ 1,180.00 </v>
+        <v>-$ 1,260.00 </v>
       </c>
       <c r="C129">
         <v>200.0</v>
@@ -2869,11 +2869,11 @@
       </c>
       <c r="E129" s="14" t="str">
         <f>A129</f>
-        <v>-$ 1,764.00 </v>
+        <v>-$ 1,836.00 </v>
       </c>
       <c r="F129" s="14" t="str">
         <f>(B129+A129)</f>
-        <v>-$ 2,944.00 </v>
+        <v>-$ 3,096.00 </v>
       </c>
       <c r="G129" t="str">
         <f>IF(F129&gt;0, "TRADE","H")</f>
@@ -2912,11 +2912,11 @@
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B133" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C133">
         <v>600.0</v>
@@ -2929,11 +2929,11 @@
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="4" t="str">
         <f>(A133-A132)*C133</f>
-        <v>-1752</v>
+        <v>-1824</v>
       </c>
       <c r="B134" s="14" t="str">
         <f>C134*(B132-B133)</f>
-        <v>-$ 1,640.00 </v>
+        <v>-$ 1,720.00 </v>
       </c>
       <c r="C134">
         <v>200.0</v>
@@ -2943,11 +2943,11 @@
       </c>
       <c r="E134" s="14" t="str">
         <f>A134</f>
-        <v>-$ 1,752.00 </v>
+        <v>-$ 1,824.00 </v>
       </c>
       <c r="F134" s="14" t="str">
         <f>(B134+A134)</f>
-        <v>-$ 3,392.00 </v>
+        <v>-$ 3,544.00 </v>
       </c>
       <c r="G134" t="str">
         <f>IF(F134&gt;0, "TRADE","H")</f>
@@ -2986,11 +2986,11 @@
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B138" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C138">
         <v>600.0</v>
@@ -3003,11 +3003,11 @@
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="4" t="str">
         <f>(A138-A137)*C138</f>
-        <v>-1944</v>
+        <v>-2016</v>
       </c>
       <c r="B139" s="14" t="str">
         <f>C139*(B137-B138)</f>
-        <v>-$ 1,590.00 </v>
+        <v>-$ 1,670.00 </v>
       </c>
       <c r="C139">
         <v>200.0</v>
@@ -3017,11 +3017,11 @@
       </c>
       <c r="E139" s="14" t="str">
         <f>A139</f>
-        <v>-$ 1,944.00 </v>
+        <v>-$ 2,016.00 </v>
       </c>
       <c r="F139" s="14" t="str">
         <f>(B139+A139)</f>
-        <v>-$ 3,534.00 </v>
+        <v>-$ 3,686.00 </v>
       </c>
       <c r="G139" t="str">
         <f>IF(F139&gt;0, "TRADE","H")</f>
@@ -3062,11 +3062,11 @@
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.60 </v>
+        <v> $ 22.48 </v>
       </c>
       <c r="B143" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 64.70 </v>
+        <v> $ 65.10 </v>
       </c>
       <c r="C143">
         <v>600.0</v>
@@ -3079,11 +3079,11 @@
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="4" t="str">
         <f>(A143-A142)*C143</f>
-        <v>-4410</v>
+        <v>-4482</v>
       </c>
       <c r="B144" s="14" t="str">
         <f>C144*(B142-B143)</f>
-        <v> $ 30.80 </v>
+        <v>-$ 49.20 </v>
       </c>
       <c r="C144">
         <v>200.0</v>
@@ -3093,11 +3093,11 @@
       </c>
       <c r="E144" s="14" t="str">
         <f>A144</f>
-        <v>-$ 4,410.00 </v>
+        <v>-$ 4,482.00 </v>
       </c>
       <c r="F144" s="14" t="str">
         <f>(B144+A144)</f>
-        <v>-$ 4,379.20 </v>
+        <v>-$ 4,531.20 </v>
       </c>
       <c r="G144" t="str">
         <f>IF(F144&gt;0, "TRADE","H")</f>
@@ -3116,7 +3116,7 @@
       <c r="F145" s="5"/>
       <c r="H145" s="5" t="str">
         <f t="shared" ref="H145:H146" si="7">(I145-K145)/K145-$D$3</f>
-        <v>-2.69%</v>
+        <v>-2.28%</v>
       </c>
       <c r="I145" s="9">
         <v>394.0</v>
@@ -3139,7 +3139,7 @@
       <c r="F146" s="5"/>
       <c r="H146" s="5" t="str">
         <f t="shared" si="7"/>
-        <v>-3.66%</v>
+        <v>-3.25%</v>
       </c>
       <c r="I146" s="11">
         <v>25.54</v>
@@ -3364,10 +3364,10 @@
       </c>
       <c r="H160" s="5" t="str">
         <f t="shared" ref="H160:H161" si="8">(I160-K160)/K160-$D$3</f>
-        <v>-3.94%</v>
+        <v>-4.28%</v>
       </c>
       <c r="I160" s="11">
-        <v>81.15</v>
+        <v>80.5</v>
       </c>
       <c r="J160" s="12">
         <v>1211.0</v>
@@ -3386,10 +3386,10 @@
       </c>
       <c r="H161" s="5" t="str">
         <f t="shared" si="8"/>
-        <v>-4.28%</v>
+        <v>-6.00%</v>
       </c>
       <c r="I161" s="11">
-        <v>89.2</v>
+        <v>87.15</v>
       </c>
       <c r="J161" s="12" t="s">
         <v>10</v>
@@ -3411,11 +3411,11 @@
     <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="15" t="str">
         <f>byd</f>
-        <v> $ 81.15 </v>
+        <v> $ 80.50 </v>
       </c>
       <c r="B163" s="15" t="str">
         <f>I161</f>
-        <v> $ 89.20 </v>
+        <v> $ 87.15 </v>
       </c>
       <c r="C163">
         <v>300.0</v>
@@ -3488,11 +3488,11 @@
     <row r="168" ht="15.75" customHeight="1">
       <c r="A168" s="14" t="str">
         <f>$B$163</f>
-        <v> $ 89.20 </v>
+        <v> $ 87.15 </v>
       </c>
       <c r="B168" s="14" t="str">
         <f>$A$163</f>
-        <v> $ 81.15 </v>
+        <v> $ 80.50 </v>
       </c>
       <c r="C168">
         <v>300.0</v>
@@ -3507,11 +3507,11 @@
     <row r="169" ht="15.75" customHeight="1">
       <c r="A169" s="14" t="str">
         <f>C169*(A168-A167)</f>
-        <v>-$ 5,070.00 </v>
+        <v>-$ 5,685.00 </v>
       </c>
       <c r="B169" s="14" t="str">
         <f>C168*(B167-B168)</f>
-        <v> $ 3,375.00 </v>
+        <v> $ 3,570.00 </v>
       </c>
       <c r="C169">
         <v>300.0</v>
@@ -3521,11 +3521,11 @@
       </c>
       <c r="E169" s="14" t="str">
         <f>A169</f>
-        <v>-$ 5,070.00 </v>
+        <v>-$ 5,685.00 </v>
       </c>
       <c r="F169" s="14" t="str">
         <f>(B169+A169)</f>
-        <v>-$ 1,695.00 </v>
+        <v>-$ 2,115.00 </v>
       </c>
       <c r="G169" t="str">
         <f>IF(F169&gt;0, "TRADE","H")</f>
@@ -3571,11 +3571,11 @@
     <row r="173" ht="15.75" customHeight="1">
       <c r="A173" s="14" t="str">
         <f>$A$163</f>
-        <v> $ 81.15 </v>
+        <v> $ 80.50 </v>
       </c>
       <c r="B173" s="14" t="str">
         <f>$B$163</f>
-        <v> $ 89.20 </v>
+        <v> $ 87.15 </v>
       </c>
       <c r="C173">
         <v>300.0</v>
@@ -3590,11 +3590,11 @@
     <row r="174" ht="15.75" customHeight="1">
       <c r="A174" s="14" t="str">
         <f>C174*(A173-A172)</f>
-        <v>-$ 1,320.00 </v>
+        <v>-$ 1,515.00 </v>
       </c>
       <c r="B174" s="14" t="str">
         <f>C173*(B172-B173)</f>
-        <v> $ 645.00 </v>
+        <v> $ 1,260.00 </v>
       </c>
       <c r="C174">
         <v>300.0</v>
@@ -3604,11 +3604,11 @@
       </c>
       <c r="E174" s="14" t="str">
         <f>A174</f>
-        <v>-$ 1,320.00 </v>
+        <v>-$ 1,515.00 </v>
       </c>
       <c r="F174" s="14" t="str">
         <f>(B174+A174)</f>
-        <v>-$ 675.00 </v>
+        <v>-$ 255.00 </v>
       </c>
       <c r="G174" t="str">
         <f>IF(F174&gt;0, "TRADE","H")</f>
@@ -3654,11 +3654,11 @@
     <row r="178" ht="15.75" customHeight="1">
       <c r="A178" s="14" t="str">
         <f>$A$163</f>
-        <v> $ 81.15 </v>
+        <v> $ 80.50 </v>
       </c>
       <c r="B178" s="14" t="str">
         <f>$B$163</f>
-        <v> $ 89.20 </v>
+        <v> $ 87.15 </v>
       </c>
       <c r="C178">
         <v>300.0</v>
@@ -3673,11 +3673,11 @@
     <row r="179" ht="15.75" customHeight="1">
       <c r="A179" s="14" t="str">
         <f>C179*(A178-A177)</f>
-        <v>-$ 3,330.00 </v>
+        <v>-$ 3,525.00 </v>
       </c>
       <c r="B179" s="14" t="str">
         <f>C178*(B177-B178)</f>
-        <v> $ 1,635.00 </v>
+        <v> $ 2,250.00 </v>
       </c>
       <c r="C179">
         <v>300.0</v>
@@ -3687,11 +3687,11 @@
       </c>
       <c r="E179" s="14" t="str">
         <f>A179</f>
-        <v>-$ 3,330.00 </v>
+        <v>-$ 3,525.00 </v>
       </c>
       <c r="F179" s="14" t="str">
         <f>(B179+A179)</f>
-        <v>-$ 1,695.00 </v>
+        <v>-$ 1,275.00 </v>
       </c>
       <c r="G179" t="str">
         <f>IF(F179&gt;0, "TRADE","H")</f>
@@ -3801,11 +3801,11 @@
     <row r="183" ht="15.75" customHeight="1">
       <c r="A183" s="23" t="str">
         <f>$B$163</f>
-        <v> $ 89.20 </v>
+        <v> $ 87.15 </v>
       </c>
       <c r="B183" s="23" t="str">
         <f>$A$163</f>
-        <v> $ 81.15 </v>
+        <v> $ 80.50 </v>
       </c>
       <c r="C183" s="19">
         <v>300.0</v>
@@ -3839,11 +3839,11 @@
     <row r="184" ht="15.75" customHeight="1">
       <c r="A184" s="23" t="str">
         <f>C184*(A183-A182)</f>
-        <v>-$ 4,650.00 </v>
+        <v>-$ 5,265.00 </v>
       </c>
       <c r="B184" s="23" t="str">
         <f>C183*(B182-B183)</f>
-        <v> $ 1,050.00 </v>
+        <v> $ 1,245.00 </v>
       </c>
       <c r="C184" s="19">
         <v>300.0</v>
@@ -3853,11 +3853,11 @@
       </c>
       <c r="E184" s="23" t="str">
         <f>A184</f>
-        <v>-$ 4,650.00 </v>
+        <v>-$ 5,265.00 </v>
       </c>
       <c r="F184" s="23" t="str">
         <f>(B184+A184)</f>
-        <v>-$ 3,600.00 </v>
+        <v>-$ 4,020.00 </v>
       </c>
       <c r="G184" s="19" t="str">
         <f>IF(F184&gt;0, "TRADE","H")</f>
@@ -3984,11 +3984,11 @@
     <row r="188" ht="15.75" customHeight="1">
       <c r="A188" s="23" t="str">
         <f>$B$163</f>
-        <v> $ 89.20 </v>
+        <v> $ 87.15 </v>
       </c>
       <c r="B188" s="23" t="str">
         <f>$A$163</f>
-        <v> $ 81.15 </v>
+        <v> $ 80.50 </v>
       </c>
       <c r="C188" s="19">
         <v>300.0</v>
@@ -4022,11 +4022,11 @@
     <row r="189" ht="15.75" customHeight="1">
       <c r="A189" s="23" t="str">
         <f>C189*(A188-A187)</f>
-        <v>-$ 5,970.00 </v>
+        <v>-$ 6,585.00 </v>
       </c>
       <c r="B189" s="23" t="str">
         <f>C188*(B187-B188)</f>
-        <v> $ 735.00 </v>
+        <v> $ 930.00 </v>
       </c>
       <c r="C189" s="19">
         <v>300.0</v>
@@ -4036,11 +4036,11 @@
       </c>
       <c r="E189" s="23" t="str">
         <f>A189</f>
-        <v>-$ 5,970.00 </v>
+        <v>-$ 6,585.00 </v>
       </c>
       <c r="F189" s="23" t="str">
         <f>(B189+A189)</f>
-        <v>-$ 5,235.00 </v>
+        <v>-$ 5,655.00 </v>
       </c>
       <c r="G189" s="19" t="str">
         <f>IF(F189&gt;0, "TRADE","H")</f>
@@ -4078,10 +4078,10 @@
       </c>
       <c r="H190" s="5" t="str">
         <f t="shared" ref="H190:H191" si="9">(I190-K190)/K190-$D$3</f>
-        <v>-5.53%</v>
+        <v>-4.71%</v>
       </c>
       <c r="I190" s="9">
-        <v>15.55</v>
+        <v>15.62</v>
       </c>
       <c r="J190" s="10">
         <v>6680.0</v>
@@ -4099,10 +4099,10 @@
       </c>
       <c r="H191" s="5" t="str">
         <f t="shared" si="9"/>
-        <v>-4.17%</v>
+        <v>-4.79%</v>
       </c>
       <c r="I191" s="11">
-        <v>80.95</v>
+        <v>80.05</v>
       </c>
       <c r="J191" s="12">
         <v>1211.0</v>
@@ -4121,17 +4121,17 @@
       </c>
       <c r="H192" s="5" t="str">
         <f>H190-H191</f>
-        <v>-1.36%</v>
+        <v>0.08%</v>
       </c>
     </row>
     <row r="193" ht="15.75" customHeight="1">
       <c r="A193" s="15" t="str">
         <f>I190</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="B193" s="15" t="str">
         <f>I191</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="C193">
         <v>800.0</v>
@@ -4197,11 +4197,11 @@
     <row r="198" ht="15.75" customHeight="1">
       <c r="A198" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="B198" s="14" t="str">
         <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="C198" s="17">
         <v>800.0</v>
@@ -4214,11 +4214,11 @@
     <row r="199" ht="15.75" customHeight="1">
       <c r="A199" s="4" t="str">
         <f>(A198-A197)*C198</f>
-        <v>-8337.52</v>
+        <v>-8281.52</v>
       </c>
       <c r="B199" s="14" t="str">
         <f>C199*(B197-B198)</f>
-        <v> $ 5,008.00 </v>
+        <v> $ 5,188.00 </v>
       </c>
       <c r="C199" s="17">
         <v>200.0</v>
@@ -4228,11 +4228,11 @@
       </c>
       <c r="E199" s="14" t="str">
         <f>A199</f>
-        <v>-$ 8,337.52 </v>
+        <v>-$ 8,281.52 </v>
       </c>
       <c r="F199" s="14" t="str">
         <f>(B199+A199)</f>
-        <v>-$ 3,329.52 </v>
+        <v>-$ 3,093.52 </v>
       </c>
       <c r="G199" t="str">
         <f>IF(F199&gt;0, "TRADE","H")</f>
@@ -4271,11 +4271,11 @@
     <row r="203" ht="15.75" customHeight="1">
       <c r="A203" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="B203" s="14" t="str">
         <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="C203" s="17">
         <v>800.0</v>
@@ -4288,11 +4288,11 @@
     <row r="204" ht="15.75" customHeight="1">
       <c r="A204" s="4" t="str">
         <f>(A203-A202)*C203</f>
-        <v>-2560</v>
+        <v>-2504</v>
       </c>
       <c r="B204" s="14" t="str">
         <f>C204*(B202-B203)</f>
-        <v> $ 130.00 </v>
+        <v> $ 310.00 </v>
       </c>
       <c r="C204" s="17">
         <v>200.0</v>
@@ -4302,11 +4302,11 @@
       </c>
       <c r="E204" s="14" t="str">
         <f>A204</f>
-        <v>-$ 2,560.00 </v>
+        <v>-$ 2,504.00 </v>
       </c>
       <c r="F204" s="14" t="str">
         <f>(B204+A204)</f>
-        <v>-$ 2,430.00 </v>
+        <v>-$ 2,194.00 </v>
       </c>
       <c r="G204" t="str">
         <f>IF(F204&gt;0, "TRADE","H")</f>
@@ -4345,11 +4345,11 @@
     <row r="208" ht="15.75" customHeight="1">
       <c r="A208" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="B208" s="14" t="str">
         <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="C208" s="26">
         <v>1200.0</v>
@@ -4362,11 +4362,11 @@
     <row r="209" ht="15.75" customHeight="1">
       <c r="A209" s="4" t="str">
         <f>(A208-A207)*C208</f>
-        <v>-2892</v>
+        <v>-2808</v>
       </c>
       <c r="B209" s="14" t="str">
         <f>C209*(B207-B208)</f>
-        <v> $ 1,050.00 </v>
+        <v> $ 1,320.00 </v>
       </c>
       <c r="C209" s="26">
         <v>300.0</v>
@@ -4376,11 +4376,11 @@
       </c>
       <c r="E209" s="14" t="str">
         <f>A209</f>
-        <v>-$ 2,892.00 </v>
+        <v>-$ 2,808.00 </v>
       </c>
       <c r="F209" s="14" t="str">
         <f>(B209+A209)</f>
-        <v>-$ 1,842.00 </v>
+        <v>-$ 1,488.00 </v>
       </c>
       <c r="G209" t="str">
         <f>IF(F209&gt;0, "TRADE","H")</f>
@@ -4419,11 +4419,11 @@
     <row r="213" ht="15.75" customHeight="1">
       <c r="A213" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="B213" s="14" t="str">
         <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="C213" s="26">
         <v>1200.0</v>
@@ -4436,11 +4436,11 @@
     <row r="214" ht="15.75" customHeight="1">
       <c r="A214" s="4" t="str">
         <f>(A213-A212)*C213</f>
-        <v>-2772</v>
+        <v>-2688</v>
       </c>
       <c r="B214" s="14" t="str">
         <f>C214*(B212-B213)</f>
-        <v> $ 1,200.00 </v>
+        <v> $ 1,470.00 </v>
       </c>
       <c r="C214" s="26">
         <v>300.0</v>
@@ -4450,11 +4450,11 @@
       </c>
       <c r="E214" s="14" t="str">
         <f>A214</f>
-        <v>-$ 2,772.00 </v>
+        <v>-$ 2,688.00 </v>
       </c>
       <c r="F214" s="14" t="str">
         <f>(B214+A214)</f>
-        <v>-$ 1,572.00 </v>
+        <v>-$ 1,218.00 </v>
       </c>
       <c r="G214" t="str">
         <f>IF(F214&gt;0, "TRADE","H")</f>
@@ -4493,11 +4493,11 @@
     <row r="218" ht="15.75" customHeight="1">
       <c r="A218" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="B218" s="14" t="str">
         <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="C218" s="17">
         <v>800.0</v>
@@ -4510,11 +4510,11 @@
     <row r="219" ht="15.75" customHeight="1">
       <c r="A219" s="4" t="str">
         <f>(A218-A217)*C218</f>
-        <v>-1536</v>
+        <v>-1480</v>
       </c>
       <c r="B219" s="14" t="str">
         <f>C219*(B217-B218)</f>
-        <v> $ 940.00 </v>
+        <v> $ 1,120.00 </v>
       </c>
       <c r="C219" s="17">
         <v>200.0</v>
@@ -4524,11 +4524,11 @@
       </c>
       <c r="E219" s="14" t="str">
         <f>A219</f>
-        <v>-$ 1,536.00 </v>
+        <v>-$ 1,480.00 </v>
       </c>
       <c r="F219" s="14" t="str">
         <f>(B219+A219)</f>
-        <v>-$ 596.00 </v>
+        <v>-$ 360.00 </v>
       </c>
       <c r="G219" t="str">
         <f>IF(F219&gt;0, "TRADE","H")</f>
@@ -4567,11 +4567,11 @@
     <row r="223" ht="15.75" customHeight="1">
       <c r="A223" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="B223" s="14" t="str">
         <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="C223" s="17">
         <v>800.0</v>
@@ -4584,11 +4584,11 @@
     <row r="224" ht="15.75" customHeight="1">
       <c r="A224" s="4" t="str">
         <f>(A223-A222)*C223</f>
-        <v>-432</v>
+        <v>-376</v>
       </c>
       <c r="B224" s="14" t="str">
         <f>C224*(B222-B223)</f>
-        <v> $ 90.00 </v>
+        <v> $ 270.00 </v>
       </c>
       <c r="C224" s="17">
         <v>200.0</v>
@@ -4598,11 +4598,11 @@
       </c>
       <c r="E224" s="14" t="str">
         <f>A224</f>
-        <v>-$ 432.00 </v>
+        <v>-$ 376.00 </v>
       </c>
       <c r="F224" s="14" t="str">
         <f>(B224+A224)</f>
-        <v>-$ 342.00 </v>
+        <v>-$ 106.00 </v>
       </c>
       <c r="G224" t="str">
         <f>IF(F224&gt;0, "TRADE","H")</f>
@@ -4618,37 +4618,37 @@
         <v>6</v>
       </c>
       <c r="C225" s="8">
-        <v>46288.0</v>
+        <v>46289.0</v>
       </c>
     </row>
     <row r="226" ht="15.75" customHeight="1">
       <c r="A226" s="4">
+        <v>1211.0</v>
+      </c>
+      <c r="B226" s="4">
         <v>6680.0</v>
-      </c>
-      <c r="B226" s="4">
-        <v>1211.0</v>
       </c>
       <c r="M226" s="6"/>
     </row>
     <row r="227" ht="15.75" customHeight="1">
       <c r="A227" s="13">
-        <v>15.55</v>
+        <v>80.05</v>
       </c>
       <c r="B227" s="14">
-        <v>80.95</v>
+        <v>15.62</v>
       </c>
     </row>
     <row r="228" ht="15.75" customHeight="1">
       <c r="A228" s="14" t="str">
+        <f>$B$193</f>
+        <v> $ 80.05 </v>
+      </c>
+      <c r="B228" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
-      </c>
-      <c r="B228" s="14" t="str">
-        <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="C228" s="17">
-        <v>800.0</v>
+        <v>200.0</v>
       </c>
       <c r="D228" t="s">
         <v>8</v>
@@ -4665,7 +4665,7 @@
         <v> $ -   </v>
       </c>
       <c r="C229" s="17">
-        <v>200.0</v>
+        <v>800.0</v>
       </c>
       <c r="D229" t="s">
         <v>9</v>
@@ -4715,11 +4715,11 @@
     <row r="233" ht="15.75" customHeight="1">
       <c r="A233" s="14" t="str">
         <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="B233" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="C233" s="17">
         <v>200.0</v>
@@ -4732,11 +4732,11 @@
     <row r="234" ht="15.75" customHeight="1">
       <c r="A234" s="4" t="str">
         <f>(A233-A232)*C233</f>
-        <v>-760</v>
+        <v>-940</v>
       </c>
       <c r="B234" s="14" t="str">
         <f>C234*(B232-B233)</f>
-        <v> $ 560.00 </v>
+        <v> $ 504.00 </v>
       </c>
       <c r="C234" s="17">
         <v>800.0</v>
@@ -4746,11 +4746,11 @@
       </c>
       <c r="E234" s="14" t="str">
         <f>A234</f>
-        <v>-$ 760.00 </v>
+        <v>-$ 940.00 </v>
       </c>
       <c r="F234" s="14" t="str">
         <f>(B234+A234)</f>
-        <v>-$ 200.00 </v>
+        <v>-$ 436.00 </v>
       </c>
       <c r="G234" t="str">
         <f>IF(F234&gt;0, "TRADE","H")</f>
@@ -4789,11 +4789,11 @@
     <row r="238" ht="15.75" customHeight="1">
       <c r="A238" s="14" t="str">
         <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="B238" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="C238" s="26">
         <v>300.0</v>
@@ -4806,11 +4806,11 @@
     <row r="239" ht="15.75" customHeight="1">
       <c r="A239" s="4" t="str">
         <f>(A238-A237)*C238</f>
-        <v>-2265</v>
+        <v>-2535</v>
       </c>
       <c r="B239" s="14" t="str">
         <f>C239*(B237-B238)</f>
-        <v> $ 1,704.00 </v>
+        <v> $ 1,620.00 </v>
       </c>
       <c r="C239" s="26">
         <v>1200.0</v>
@@ -4820,11 +4820,11 @@
       </c>
       <c r="E239" s="14" t="str">
         <f>A239</f>
-        <v>-$ 2,265.00 </v>
+        <v>-$ 2,535.00 </v>
       </c>
       <c r="F239" s="14" t="str">
         <f>(B239+A239)</f>
-        <v>-$ 561.00 </v>
+        <v>-$ 915.00 </v>
       </c>
       <c r="G239" t="str">
         <f>IF(F239&gt;0, "TRADE","H")</f>
@@ -4863,11 +4863,11 @@
     <row r="243" ht="15.75" customHeight="1">
       <c r="A243" s="14" t="str">
         <f>$B$193</f>
-        <v> $ 80.95 </v>
+        <v> $ 80.05 </v>
       </c>
       <c r="B243" s="14" t="str">
         <f>$A$193</f>
-        <v> $ 15.55 </v>
+        <v> $ 15.62 </v>
       </c>
       <c r="C243" s="17">
         <v>200.0</v>
@@ -4880,11 +4880,11 @@
     <row r="244" ht="15.75" customHeight="1">
       <c r="A244" s="4" t="str">
         <f>(A243-A242)*C243</f>
-        <v>-2060</v>
+        <v>-2240</v>
       </c>
       <c r="B244" s="14" t="str">
         <f>C244*(B242-B243)</f>
-        <v> $ 1,344.00 </v>
+        <v> $ 1,288.00 </v>
       </c>
       <c r="C244" s="17">
         <v>800.0</v>
@@ -4894,11 +4894,11 @@
       </c>
       <c r="E244" s="14" t="str">
         <f>A244</f>
-        <v>-$ 2,060.00 </v>
+        <v>-$ 2,240.00 </v>
       </c>
       <c r="F244" s="14" t="str">
         <f>(B244+A244)</f>
-        <v>-$ 716.00 </v>
+        <v>-$ 952.00 </v>
       </c>
       <c r="G244" t="str">
         <f>IF(F244&gt;0, "TRADE","H")</f>
@@ -4914,7 +4914,7 @@
       <c r="E245" s="14"/>
       <c r="H245" s="5" t="str">
         <f t="shared" ref="H245:H246" si="10">(I245-K245)/K245-$D$3</f>
-        <v>5.10%</v>
+        <v>5.51%</v>
       </c>
       <c r="I245" s="9">
         <v>0.194</v>
@@ -4939,7 +4939,7 @@
       </c>
       <c r="H246" s="5" t="str">
         <f t="shared" si="10"/>
-        <v>0.52%</v>
+        <v>0.93%</v>
       </c>
       <c r="I246" s="11">
         <v>0.59</v>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="H261" s="5" t="str">
         <f t="shared" ref="H261:H262" si="11">(I261-K261)/K261-$D$3</f>
-        <v>11.42%</v>
+        <v>11.83%</v>
       </c>
       <c r="I261" s="9">
         <v>104.3</v>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="H262" s="5" t="str">
         <f t="shared" si="11"/>
-        <v>1.19%</v>
+        <v>1.60%</v>
       </c>
       <c r="I262" s="11">
         <v>444.8</v>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="H266" s="5" t="str">
         <f t="shared" ref="H266:H267" si="12">(I266-K266)/K266-$D$3</f>
-        <v>-11.92%</v>
+        <v>-11.51%</v>
       </c>
       <c r="I266" s="11">
         <v>23.28</v>
@@ -5297,7 +5297,7 @@
       </c>
       <c r="H267" s="5" t="str">
         <f t="shared" si="12"/>
-        <v>48.53%</v>
+        <v>48.94%</v>
       </c>
       <c r="I267" s="11">
         <v>140.0</v>
@@ -5453,10 +5453,10 @@
       </c>
       <c r="H276" s="5" t="str">
         <f t="shared" ref="H276:H277" si="14">(I276-K276)/K276-$D$3</f>
-        <v>-5.93%</v>
+        <v>-4.82%</v>
       </c>
       <c r="I276" s="9">
-        <v>64.75</v>
+        <v>65.25</v>
       </c>
       <c r="J276" s="10">
         <v>2382.0</v>
@@ -5475,10 +5475,10 @@
       </c>
       <c r="H277" s="5" t="str">
         <f t="shared" si="14"/>
-        <v>-4.54%</v>
+        <v>-6.21%</v>
       </c>
       <c r="I277" s="9">
-        <v>88.95</v>
+        <v>86.95</v>
       </c>
       <c r="J277" s="12" t="s">
         <v>10</v>
@@ -5496,7 +5496,7 @@
       </c>
       <c r="H278" s="5" t="str">
         <f>H276-H277</f>
-        <v>-1.39%</v>
+        <v>1.39%</v>
       </c>
       <c r="I278" s="17"/>
       <c r="Y278" s="6"/>
@@ -5504,11 +5504,11 @@
     <row r="279" ht="15.75" customHeight="1">
       <c r="A279" s="15" t="str">
         <f>I276</f>
-        <v> $ 64.75 </v>
+        <v> $ 65.25 </v>
       </c>
       <c r="B279" s="15" t="str">
         <f>I277</f>
-        <v> $ 88.95 </v>
+        <v> $ 86.95 </v>
       </c>
       <c r="C279">
         <v>200.0</v>
@@ -5570,11 +5570,11 @@
     <row r="284" ht="15.75" customHeight="1">
       <c r="A284" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 88.95 </v>
+        <v> $ 86.95 </v>
       </c>
       <c r="B284" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 64.75 </v>
+        <v> $ 65.25 </v>
       </c>
       <c r="C284">
         <v>200.0</v>
@@ -5585,22 +5585,22 @@
     <row r="285" ht="15.75" customHeight="1">
       <c r="A285" s="4" t="str">
         <f>(A284-A283)*C285</f>
-        <v>-950</v>
+        <v>-1350</v>
       </c>
       <c r="B285" s="4" t="str">
         <f>(B283-B284)*C284</f>
-        <v>650</v>
+        <v>550</v>
       </c>
       <c r="C285">
         <v>200.0</v>
       </c>
       <c r="E285" s="14" t="str">
         <f>A285</f>
-        <v>-$ 950.00 </v>
+        <v>-$ 1,350.00 </v>
       </c>
       <c r="F285" s="4" t="str">
         <f>(B285+A285)</f>
-        <v>-300</v>
+        <v>-800</v>
       </c>
       <c r="G285" t="str">
         <f>IF(F285&gt;0, "TRADE","H")</f>
@@ -5645,11 +5645,11 @@
     <row r="289" ht="15.75" customHeight="1">
       <c r="A289" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 64.75 </v>
+        <v> $ 65.25 </v>
       </c>
       <c r="B289" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 88.95 </v>
+        <v> $ 86.95 </v>
       </c>
       <c r="C289">
         <v>200.0</v>
@@ -5660,26 +5660,26 @@
     <row r="290" ht="15.75" customHeight="1">
       <c r="A290" s="4" t="str">
         <f>(A289-A288)*C290</f>
-        <v>-450</v>
+        <v>-350</v>
       </c>
       <c r="B290" s="4" t="str">
         <f>(B288-B289)*C289</f>
-        <v>110</v>
+        <v>510</v>
       </c>
       <c r="C290">
         <v>200.0</v>
       </c>
       <c r="E290" s="14" t="str">
         <f>A290</f>
-        <v>-$ 450.00 </v>
+        <v>-$ 350.00 </v>
       </c>
       <c r="F290" s="4" t="str">
         <f>(B290+A290)</f>
-        <v>-340</v>
+        <v>160</v>
       </c>
       <c r="G290" t="str">
         <f>IF(F290&gt;0, "TRADE","H")</f>
-        <v>H</v>
+        <v>TRADE</v>
       </c>
       <c r="H290" s="5"/>
       <c r="N290" s="6"/>
@@ -5721,11 +5721,11 @@
     <row r="294" ht="15.75" customHeight="1">
       <c r="A294" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 64.75 </v>
+        <v> $ 65.25 </v>
       </c>
       <c r="B294" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 88.95 </v>
+        <v> $ 86.95 </v>
       </c>
       <c r="C294">
         <v>200.0</v>
@@ -5736,22 +5736,22 @@
     <row r="295" ht="15.75" customHeight="1">
       <c r="A295" s="4" t="str">
         <f>(A294-A293)*C295</f>
-        <v>-3538.8</v>
+        <v>-3438.8</v>
       </c>
       <c r="B295" s="4" t="str">
         <f>(B293-B294)*C294</f>
-        <v>990</v>
+        <v>1390</v>
       </c>
       <c r="C295">
         <v>200.0</v>
       </c>
       <c r="E295" s="14" t="str">
         <f>A295</f>
-        <v>-$ 3,538.80 </v>
+        <v>-$ 3,438.80 </v>
       </c>
       <c r="F295" s="4" t="str">
         <f>(B295+A295)</f>
-        <v>-2548.8</v>
+        <v>-2048.8</v>
       </c>
       <c r="G295" t="str">
         <f>IF(F295&gt;0, "TRADE","H")</f>
@@ -5797,11 +5797,11 @@
     <row r="299" ht="15.75" customHeight="1">
       <c r="A299" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 64.75 </v>
+        <v> $ 65.25 </v>
       </c>
       <c r="B299" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 88.95 </v>
+        <v> $ 86.95 </v>
       </c>
       <c r="C299">
         <v>200.0</v>
@@ -5812,22 +5812,22 @@
     <row r="300" ht="15.75" customHeight="1">
       <c r="A300" s="4" t="str">
         <f>(A299-A298)*C300</f>
-        <v>-3518.8</v>
+        <v>-3418.8</v>
       </c>
       <c r="B300" s="4" t="str">
         <f>(B298-B299)*C299</f>
-        <v>150</v>
+        <v>550</v>
       </c>
       <c r="C300">
         <v>200.0</v>
       </c>
       <c r="E300" s="14" t="str">
         <f>A300</f>
-        <v>-$ 3,518.80 </v>
+        <v>-$ 3,418.80 </v>
       </c>
       <c r="F300" s="4" t="str">
         <f>(B300+A300)</f>
-        <v>-3368.8</v>
+        <v>-2868.8</v>
       </c>
       <c r="G300" t="str">
         <f>IF(F300&gt;0, "TRADE","H")</f>
@@ -5873,11 +5873,11 @@
     <row r="304" ht="15.75" customHeight="1">
       <c r="A304" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 64.75 </v>
+        <v> $ 65.25 </v>
       </c>
       <c r="B304" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 88.95 </v>
+        <v> $ 86.95 </v>
       </c>
       <c r="C304">
         <v>200.0</v>
@@ -5888,22 +5888,22 @@
     <row r="305" ht="15.75" customHeight="1">
       <c r="A305" s="4" t="str">
         <f>(A304-A303)*C305</f>
-        <v>-3208.8</v>
+        <v>-3108.8</v>
       </c>
       <c r="B305" s="4" t="str">
         <f>(B303-B304)*C304</f>
-        <v>-210</v>
+        <v>190</v>
       </c>
       <c r="C305">
         <v>200.0</v>
       </c>
       <c r="E305" s="14" t="str">
         <f>A305</f>
-        <v>-$ 3,208.80 </v>
+        <v>-$ 3,108.80 </v>
       </c>
       <c r="F305" s="4" t="str">
         <f>(B305+A305)</f>
-        <v>-3418.8</v>
+        <v>-2918.8</v>
       </c>
       <c r="G305" t="str">
         <f>IF(F305&gt;0, "TRADE","H")</f>
@@ -5949,11 +5949,11 @@
     <row r="309" ht="15.75" customHeight="1">
       <c r="A309" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 64.75 </v>
+        <v> $ 65.25 </v>
       </c>
       <c r="B309" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 88.95 </v>
+        <v> $ 86.95 </v>
       </c>
       <c r="C309">
         <v>200.0</v>
@@ -5964,22 +5964,22 @@
     <row r="310" ht="15.75" customHeight="1">
       <c r="A310" s="4" t="str">
         <f>(A309-A308)*C310</f>
-        <v>-3552.4</v>
+        <v>-3452.4</v>
       </c>
       <c r="B310" s="4" t="str">
         <f>(B308-B309)*C309</f>
-        <v>-1010</v>
+        <v>-610</v>
       </c>
       <c r="C310">
         <v>200.0</v>
       </c>
       <c r="E310" s="14" t="str">
         <f>A310</f>
-        <v>-$ 3,552.40 </v>
+        <v>-$ 3,452.40 </v>
       </c>
       <c r="F310" s="4" t="str">
         <f>(B310+A310)</f>
-        <v>-4562.4</v>
+        <v>-4062.4</v>
       </c>
       <c r="G310" t="str">
         <f>IF(F310&gt;0, "TRADE","H")</f>
@@ -6025,11 +6025,11 @@
     <row r="314" ht="15.75" customHeight="1">
       <c r="A314" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 64.75 </v>
+        <v> $ 65.25 </v>
       </c>
       <c r="B314" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 88.95 </v>
+        <v> $ 86.95 </v>
       </c>
       <c r="C314">
         <v>200.0</v>
@@ -6040,22 +6040,22 @@
     <row r="315" ht="15.75" customHeight="1">
       <c r="A315" s="4" t="str">
         <f>(A314-A313)*C315</f>
-        <v>-3552.4</v>
+        <v>-3452.4</v>
       </c>
       <c r="B315" s="4" t="str">
         <f>(B313-B314)*C314</f>
-        <v>-1010</v>
+        <v>-610</v>
       </c>
       <c r="C315">
         <v>200.0</v>
       </c>
       <c r="E315" s="14" t="str">
         <f>A315</f>
-        <v>-$ 3,552.40 </v>
+        <v>-$ 3,452.40 </v>
       </c>
       <c r="F315" s="4" t="str">
         <f>(B315+A315)</f>
-        <v>-4562.4</v>
+        <v>-4062.4</v>
       </c>
       <c r="G315" t="str">
         <f>IF(F315&gt;0, "TRADE","H")</f>
@@ -6076,10 +6076,10 @@
       </c>
       <c r="H316" s="5" t="str">
         <f t="shared" ref="H316:H317" si="15">(I316-K316)/K316-$D$3</f>
-        <v>-4.02%</v>
+        <v>-2.14%</v>
       </c>
       <c r="I316" s="9">
-        <v>78.85</v>
+        <v>80.1</v>
       </c>
       <c r="J316" s="10">
         <v>9880.0</v>
@@ -6098,10 +6098,10 @@
       </c>
       <c r="H317" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-4.80%</v>
+        <v>-6.16%</v>
       </c>
       <c r="I317" s="9">
-        <v>88.7</v>
+        <v>87.0</v>
       </c>
       <c r="J317" s="12" t="s">
         <v>10</v>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="H318" s="5" t="str">
         <f>H316-H317</f>
-        <v>0.78%</v>
+        <v>4.02%</v>
       </c>
       <c r="I318" s="17"/>
       <c r="Z318" s="6"/>
@@ -6128,11 +6128,11 @@
     <row r="319" ht="15.75" customHeight="1">
       <c r="A319" s="15" t="str">
         <f>I316</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="B319" s="15" t="str">
         <f>I317</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="C319">
         <v>200.0</v>
@@ -6146,11 +6146,11 @@
     <row r="320" ht="15.75" customHeight="1">
       <c r="A320" s="4" t="str">
         <f>(A319-A318)*C320</f>
-        <v>-11650</v>
+        <v>-11400</v>
       </c>
       <c r="B320" s="4" t="str">
         <f>(B318-B319)*C319</f>
-        <v>7280</v>
+        <v>7620</v>
       </c>
       <c r="C320">
         <v>200.0</v>
@@ -6160,11 +6160,11 @@
       </c>
       <c r="E320" s="14" t="str">
         <f>A320</f>
-        <v>-$ 11,650.00 </v>
+        <v>-$ 11,400.00 </v>
       </c>
       <c r="F320" s="4" t="str">
         <f>(B320+A320)</f>
-        <v>-4370</v>
+        <v>-3780</v>
       </c>
       <c r="G320" t="str">
         <f>IF(F320&gt;0, "TRADE","H")</f>
@@ -6209,11 +6209,11 @@
     <row r="324" ht="15.75" customHeight="1">
       <c r="A324" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="B324" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="C324">
         <v>200.0</v>
@@ -6227,11 +6227,11 @@
     <row r="325" ht="15.75" customHeight="1">
       <c r="A325" s="4" t="str">
         <f>(A324-A323)*C325</f>
-        <v>-4080</v>
+        <v>-4420</v>
       </c>
       <c r="B325" s="4" t="str">
         <f>(B323-B324)*C324</f>
-        <v>600</v>
+        <v>350</v>
       </c>
       <c r="C325">
         <v>200.0</v>
@@ -6241,11 +6241,11 @@
       </c>
       <c r="E325" s="14" t="str">
         <f>A325</f>
-        <v>-$ 4,080.00 </v>
+        <v>-$ 4,420.00 </v>
       </c>
       <c r="F325" s="4" t="str">
         <f>(B325+A325)</f>
-        <v>-3480</v>
+        <v>-4070</v>
       </c>
       <c r="G325" t="str">
         <f>IF(F325&gt;0, "TRADE","H")</f>
@@ -6290,11 +6290,11 @@
     <row r="329" ht="15.75" customHeight="1">
       <c r="A329" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="B329" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="C329">
         <v>200.0</v>
@@ -6308,11 +6308,11 @@
     <row r="330" ht="15.75" customHeight="1">
       <c r="A330" s="4" t="str">
         <f>(A329-A328)*C330</f>
-        <v>-3400</v>
+        <v>-3740</v>
       </c>
       <c r="B330" s="4" t="str">
         <f>(B328-B329)*C329</f>
-        <v>280</v>
+        <v>30</v>
       </c>
       <c r="C330">
         <v>200.0</v>
@@ -6322,11 +6322,11 @@
       </c>
       <c r="E330" s="14" t="str">
         <f>A330</f>
-        <v>-$ 3,400.00 </v>
+        <v>-$ 3,740.00 </v>
       </c>
       <c r="F330" s="4" t="str">
         <f>(B330+A330)</f>
-        <v>-3120</v>
+        <v>-3710</v>
       </c>
       <c r="G330" t="str">
         <f>IF(F330&gt;0, "TRADE","H")</f>
@@ -6371,11 +6371,11 @@
     <row r="334" ht="15.75" customHeight="1">
       <c r="A334" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="B334" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="C334">
         <v>200.0</v>
@@ -6389,11 +6389,11 @@
     <row r="335" ht="15.75" customHeight="1">
       <c r="A335" s="4" t="str">
         <f>(A334-A333)*C335</f>
-        <v>-2680</v>
+        <v>-3020</v>
       </c>
       <c r="B335" s="4" t="str">
         <f>(B333-B334)*C334</f>
-        <v>100</v>
+        <v>-150</v>
       </c>
       <c r="C335">
         <v>200.0</v>
@@ -6403,11 +6403,11 @@
       </c>
       <c r="E335" s="14" t="str">
         <f>A335</f>
-        <v>-$ 2,680.00 </v>
+        <v>-$ 3,020.00 </v>
       </c>
       <c r="F335" s="4" t="str">
         <f>(B335+A335)</f>
-        <v>-2580</v>
+        <v>-3170</v>
       </c>
       <c r="G335" t="str">
         <f>IF(F335&gt;0, "TRADE","H")</f>
@@ -6452,11 +6452,11 @@
     <row r="339" ht="15.75" customHeight="1">
       <c r="A339" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="B339" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="C339">
         <v>200.0</v>
@@ -6470,11 +6470,11 @@
     <row r="340" ht="15.75" customHeight="1">
       <c r="A340" s="4" t="str">
         <f>(A339-A338)*C340</f>
-        <v>-4220</v>
+        <v>-4560</v>
       </c>
       <c r="B340" s="4" t="str">
         <f>(B338-B339)*C339</f>
-        <v>1510</v>
+        <v>1260</v>
       </c>
       <c r="C340">
         <v>200.0</v>
@@ -6484,11 +6484,11 @@
       </c>
       <c r="E340" s="14" t="str">
         <f>A340</f>
-        <v>-$ 4,220.00 </v>
+        <v>-$ 4,560.00 </v>
       </c>
       <c r="F340" s="4" t="str">
         <f>(B340+A340)</f>
-        <v>-2710</v>
+        <v>-3300</v>
       </c>
       <c r="G340" t="str">
         <f>IF(F340&gt;0, "TRADE","H")</f>
@@ -6533,11 +6533,11 @@
     <row r="344" ht="15.75" customHeight="1">
       <c r="A344" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="B344" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="C344">
         <v>200.0</v>
@@ -6551,11 +6551,11 @@
     <row r="345" ht="15.75" customHeight="1">
       <c r="A345" s="4" t="str">
         <f>(A344-A343)*C345</f>
-        <v>-4040</v>
+        <v>-4380</v>
       </c>
       <c r="B345" s="4" t="str">
         <f>(B343-B344)*C344</f>
-        <v>1890</v>
+        <v>1640</v>
       </c>
       <c r="C345">
         <v>200.0</v>
@@ -6565,11 +6565,11 @@
       </c>
       <c r="E345" s="14" t="str">
         <f>A345</f>
-        <v>-$ 4,040.00 </v>
+        <v>-$ 4,380.00 </v>
       </c>
       <c r="F345" s="4" t="str">
         <f>(B345+A345)</f>
-        <v>-2150</v>
+        <v>-2740</v>
       </c>
       <c r="G345" t="str">
         <f>IF(F345&gt;0, "TRADE","H")</f>
@@ -6614,11 +6614,11 @@
     <row r="349" ht="15.75" customHeight="1">
       <c r="A349" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="B349" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="C349">
         <v>200.0</v>
@@ -6632,11 +6632,11 @@
     <row r="350" ht="15.75" customHeight="1">
       <c r="A350" s="4" t="str">
         <f>(A349-A348)*C350</f>
-        <v>-3360</v>
+        <v>-3700</v>
       </c>
       <c r="B350" s="4" t="str">
         <f>(B348-B349)*C349</f>
-        <v>1980</v>
+        <v>1730</v>
       </c>
       <c r="C350">
         <v>200.0</v>
@@ -6646,11 +6646,11 @@
       </c>
       <c r="E350" s="14" t="str">
         <f>A350</f>
-        <v>-$ 3,360.00 </v>
+        <v>-$ 3,700.00 </v>
       </c>
       <c r="F350" s="4" t="str">
         <f>(B350+A350)</f>
-        <v>-1380</v>
+        <v>-1970</v>
       </c>
       <c r="G350" t="str">
         <f>IF(F350&gt;0, "TRADE","H")</f>
@@ -6695,11 +6695,11 @@
     <row r="354" ht="15.75" customHeight="1">
       <c r="A354" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="B354" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="C354">
         <v>200.0</v>
@@ -6713,11 +6713,11 @@
     <row r="355" ht="15.75" customHeight="1">
       <c r="A355" s="4" t="str">
         <f>(A354-A353)*C355</f>
-        <v>-3260</v>
+        <v>-3600</v>
       </c>
       <c r="B355" s="4" t="str">
         <f>(B353-B354)*C354</f>
-        <v>2480</v>
+        <v>2230</v>
       </c>
       <c r="C355">
         <v>200.0</v>
@@ -6727,11 +6727,11 @@
       </c>
       <c r="E355" s="14" t="str">
         <f>A355</f>
-        <v>-$ 3,260.00 </v>
+        <v>-$ 3,600.00 </v>
       </c>
       <c r="F355" s="4" t="str">
         <f>(B355+A355)</f>
-        <v>-780</v>
+        <v>-1370</v>
       </c>
       <c r="G355" t="str">
         <f>IF(F355&gt;0, "TRADE","H")</f>
@@ -6776,11 +6776,11 @@
     <row r="359" ht="15.75" customHeight="1">
       <c r="A359" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="B359" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="C359">
         <v>200.0</v>
@@ -6794,11 +6794,11 @@
     <row r="360" ht="15.75" customHeight="1">
       <c r="A360" s="4" t="str">
         <f>(A359-A358)*C360</f>
-        <v>80</v>
+        <v>-260</v>
       </c>
       <c r="B360" s="4" t="str">
         <f>(B358-B359)*C359</f>
-        <v>-230</v>
+        <v>-480</v>
       </c>
       <c r="C360">
         <v>200.0</v>
@@ -6808,11 +6808,11 @@
       </c>
       <c r="E360" s="14" t="str">
         <f>A360</f>
-        <v> $ 80.00 </v>
+        <v>-$ 260.00 </v>
       </c>
       <c r="F360" s="4" t="str">
         <f>(B360+A360)</f>
-        <v>-150</v>
+        <v>-740</v>
       </c>
       <c r="G360" t="str">
         <f>IF(F360&gt;0, "TRADE","H")</f>
@@ -6857,11 +6857,11 @@
     <row r="364" ht="15.75" customHeight="1">
       <c r="A364" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="B364" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="C364">
         <v>200.0</v>
@@ -6875,11 +6875,11 @@
     <row r="365" ht="15.75" customHeight="1">
       <c r="A365" s="4" t="str">
         <f>(A364-A363)*C365</f>
-        <v>0</v>
+        <v>-340</v>
       </c>
       <c r="B365" s="4" t="str">
         <f>(B363-B364)*C364</f>
-        <v>0</v>
+        <v>-250</v>
       </c>
       <c r="C365">
         <v>200.0</v>
@@ -6889,11 +6889,11 @@
       </c>
       <c r="E365" s="14" t="str">
         <f>A365</f>
-        <v> $ -   </v>
+        <v>-$ 340.00 </v>
       </c>
       <c r="F365" s="4" t="str">
         <f>(B365+A365)</f>
-        <v>0</v>
+        <v>-590</v>
       </c>
       <c r="G365" t="str">
         <f>IF(F365&gt;0, "TRADE","H")</f>
@@ -6938,11 +6938,11 @@
     <row r="369" ht="15.75" customHeight="1">
       <c r="A369" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="B369" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="C369">
         <v>200.0</v>
@@ -6956,11 +6956,11 @@
     <row r="370" ht="15.75" customHeight="1">
       <c r="A370" s="4" t="str">
         <f>(A369-A368)*C370</f>
-        <v>-1090</v>
+        <v>-840</v>
       </c>
       <c r="B370" s="4" t="str">
         <f>(B368-B369)*C369</f>
-        <v>680</v>
+        <v>1020</v>
       </c>
       <c r="C370">
         <v>200.0</v>
@@ -6970,15 +6970,15 @@
       </c>
       <c r="E370" s="14" t="str">
         <f>A370</f>
-        <v>-$ 1,090.00 </v>
+        <v>-$ 840.00 </v>
       </c>
       <c r="F370" s="4" t="str">
         <f>(B370+A370)</f>
-        <v>-410</v>
+        <v>180</v>
       </c>
       <c r="G370" t="str">
         <f>IF(F370&gt;0, "TRADE","H")</f>
-        <v>H</v>
+        <v>TRADE</v>
       </c>
       <c r="H370" s="5"/>
       <c r="Z370" s="6"/>
@@ -7019,11 +7019,11 @@
     <row r="374" ht="15.75" customHeight="1">
       <c r="A374" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="B374" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="C374">
         <v>200.0</v>
@@ -7037,11 +7037,11 @@
     <row r="375" ht="15.75" customHeight="1">
       <c r="A375" s="4" t="str">
         <f>(A374-A373)*C375</f>
-        <v>-1200</v>
+        <v>-950</v>
       </c>
       <c r="B375" s="4" t="str">
         <f>(B373-B374)*C374</f>
-        <v>260</v>
+        <v>600</v>
       </c>
       <c r="C375">
         <v>200.0</v>
@@ -7051,11 +7051,11 @@
       </c>
       <c r="E375" s="14" t="str">
         <f>A375</f>
-        <v>-$ 1,200.00 </v>
+        <v>-$ 950.00 </v>
       </c>
       <c r="F375" s="4" t="str">
         <f>(B375+A375)</f>
-        <v>-940</v>
+        <v>-350</v>
       </c>
       <c r="G375" t="str">
         <f>IF(F375&gt;0, "TRADE","H")</f>
@@ -7100,11 +7100,11 @@
     <row r="379" ht="15.75" customHeight="1">
       <c r="A379" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="B379" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="C379">
         <v>200.0</v>
@@ -7118,11 +7118,11 @@
     <row r="380" ht="15.75" customHeight="1">
       <c r="A380" s="4" t="str">
         <f>(A379-A378)*C380</f>
-        <v>-1580</v>
+        <v>-1330</v>
       </c>
       <c r="B380" s="4" t="str">
         <f>(B378-B379)*C379</f>
-        <v>-170</v>
+        <v>170</v>
       </c>
       <c r="C380">
         <v>200.0</v>
@@ -7132,11 +7132,11 @@
       </c>
       <c r="E380" s="14" t="str">
         <f>A380</f>
-        <v>-$ 1,580.00 </v>
+        <v>-$ 1,330.00 </v>
       </c>
       <c r="F380" s="4" t="str">
         <f>(B380+A380)</f>
-        <v>-1750</v>
+        <v>-1160</v>
       </c>
       <c r="G380" t="str">
         <f>IF(F380&gt;0, "TRADE","H")</f>
@@ -7181,11 +7181,11 @@
     <row r="384" ht="15.75" customHeight="1">
       <c r="A384" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="B384" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="C384" s="27">
         <v>300.0</v>
@@ -7199,11 +7199,11 @@
     <row r="385" ht="15.75" customHeight="1">
       <c r="A385" s="4" t="str">
         <f>(A384-A383)*C385</f>
-        <v>-15165</v>
+        <v>-14790</v>
       </c>
       <c r="B385" s="4" t="str">
         <f>(B383-B384)*C384</f>
-        <v>12240</v>
+        <v>12750</v>
       </c>
       <c r="C385" s="27">
         <v>300.0</v>
@@ -7213,11 +7213,11 @@
       </c>
       <c r="E385" s="14" t="str">
         <f>A385</f>
-        <v>-$ 15,165.00 </v>
+        <v>-$ 14,790.00 </v>
       </c>
       <c r="F385" s="4" t="str">
         <f>(B385+A385)</f>
-        <v>-2925</v>
+        <v>-2040</v>
       </c>
       <c r="G385" t="str">
         <f>IF(F385&gt;0, "TRADE","H")</f>
@@ -7262,11 +7262,11 @@
     <row r="389" ht="15.75" customHeight="1">
       <c r="A389" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="B389" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="C389">
         <v>200.0</v>
@@ -7280,11 +7280,11 @@
     <row r="390" ht="15.75" customHeight="1">
       <c r="A390" s="4" t="str">
         <f>(A389-A388)*C390</f>
-        <v>-12850</v>
+        <v>-12600</v>
       </c>
       <c r="B390" s="4" t="str">
         <f>(B388-B389)*C389</f>
-        <v>8960</v>
+        <v>9300</v>
       </c>
       <c r="C390">
         <v>200.0</v>
@@ -7294,11 +7294,11 @@
       </c>
       <c r="E390" s="14" t="str">
         <f>A390</f>
-        <v>-$ 12,850.00 </v>
+        <v>-$ 12,600.00 </v>
       </c>
       <c r="F390" s="4" t="str">
         <f>(B390+A390)</f>
-        <v>-3890</v>
+        <v>-3300</v>
       </c>
       <c r="G390" t="str">
         <f>IF(F390&gt;0, "TRADE","H")</f>
@@ -7343,11 +7343,11 @@
     <row r="394" ht="15.75" customHeight="1">
       <c r="A394" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="B394" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="C394">
         <v>200.0</v>
@@ -7361,11 +7361,11 @@
     <row r="395" ht="15.75" customHeight="1">
       <c r="A395" s="4" t="str">
         <f>(A394-A393)*C395</f>
-        <v>-12990</v>
+        <v>-12740</v>
       </c>
       <c r="B395" s="4" t="str">
         <f>(B393-B394)*C394</f>
-        <v>8820</v>
+        <v>9160</v>
       </c>
       <c r="C395">
         <v>200.0</v>
@@ -7375,11 +7375,11 @@
       </c>
       <c r="E395" s="14" t="str">
         <f>A395</f>
-        <v>-$ 12,990.00 </v>
+        <v>-$ 12,740.00 </v>
       </c>
       <c r="F395" s="4" t="str">
         <f>(B395+A395)</f>
-        <v>-4170</v>
+        <v>-3580</v>
       </c>
       <c r="G395" t="str">
         <f>IF(F395&gt;0, "TRADE","H")</f>
@@ -7424,11 +7424,11 @@
     <row r="399" ht="15.75" customHeight="1">
       <c r="A399" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="B399" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="C399">
         <v>200.0</v>
@@ -7442,11 +7442,11 @@
     <row r="400" ht="15.75" customHeight="1">
       <c r="A400" s="4" t="str">
         <f>(A399-A398)*C400</f>
-        <v>-13150</v>
+        <v>-12900</v>
       </c>
       <c r="B400" s="4" t="str">
         <f>(B398-B399)*C399</f>
-        <v>8300</v>
+        <v>8640</v>
       </c>
       <c r="C400">
         <v>200.0</v>
@@ -7456,11 +7456,11 @@
       </c>
       <c r="E400" s="14" t="str">
         <f>A400</f>
-        <v>-$ 13,150.00 </v>
+        <v>-$ 12,900.00 </v>
       </c>
       <c r="F400" s="4" t="str">
         <f>(B400+A400)</f>
-        <v>-4850</v>
+        <v>-4260</v>
       </c>
       <c r="G400" t="str">
         <f>IF(F400&gt;0, "TRADE","H")</f>
@@ -7505,11 +7505,11 @@
     <row r="404" ht="15.75" customHeight="1">
       <c r="A404" s="14" t="str">
         <f>$A$319</f>
-        <v> $ 78.85 </v>
+        <v> $ 80.10 </v>
       </c>
       <c r="B404" s="14" t="str">
         <f>$B$319</f>
-        <v> $ 88.70 </v>
+        <v> $ 87.00 </v>
       </c>
       <c r="C404">
         <v>200.0</v>
@@ -7523,11 +7523,11 @@
     <row r="405" ht="15.75" customHeight="1">
       <c r="A405" s="4" t="str">
         <f>(A404-A403)*C405</f>
-        <v>-13550</v>
+        <v>-13300</v>
       </c>
       <c r="B405" s="4" t="str">
         <f>(B403-B404)*C404</f>
-        <v>8160</v>
+        <v>8500</v>
       </c>
       <c r="C405">
         <v>200.0</v>
@@ -7537,11 +7537,11 @@
       </c>
       <c r="E405" s="14" t="str">
         <f>A405</f>
-        <v>-$ 13,550.00 </v>
+        <v>-$ 13,300.00 </v>
       </c>
       <c r="F405" s="4" t="str">
         <f>(B405+A405)</f>
-        <v>-5390</v>
+        <v>-4800</v>
       </c>
       <c r="G405" t="str">
         <f>IF(F405&gt;0, "TRADE","H")</f>
@@ -7562,7 +7562,7 @@
       </c>
       <c r="H406" s="5" t="str">
         <f t="shared" ref="H406:H407" si="16">(I406-K406)/K406-$D$3</f>
-        <v>-48.75%</v>
+        <v>-48.34%</v>
       </c>
       <c r="I406" s="9">
         <v>0.83</v>
@@ -7582,7 +7582,7 @@
       <c r="B407" s="4"/>
       <c r="H407" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>9.08%</v>
+        <v>9.49%</v>
       </c>
       <c r="I407" s="9">
         <v>5.58</v>
@@ -9170,7 +9170,7 @@
       </c>
       <c r="H517" s="5" t="str">
         <f>(I517-K517)/K517-$D$3</f>
-        <v>81.10%</v>
+        <v>81.51%</v>
       </c>
       <c r="I517" s="9">
         <v>28.3</v>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="H527" s="5" t="str">
         <f>(I527-K527)/K527-$D$3</f>
-        <v>88.74%</v>
+        <v>89.15%</v>
       </c>
       <c r="I527" s="9">
         <v>157.7</v>
@@ -9337,7 +9337,7 @@
       <c r="B529" s="4"/>
       <c r="H529" s="5" t="str">
         <f>H527-H528</f>
-        <v>88.74%</v>
+        <v>89.15%</v>
       </c>
       <c r="Q529" s="6"/>
     </row>
@@ -18445,48 +18445,48 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
+  <conditionalFormatting sqref="F365">
     <cfRule type="cellIs" dxfId="5" priority="1768" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
+  <conditionalFormatting sqref="F365">
     <cfRule type="cellIs" dxfId="4" priority="1769" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
+  <conditionalFormatting sqref="F365">
     <cfRule type="cellIs" dxfId="4" priority="1770" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
+  <conditionalFormatting sqref="F365">
     <cfRule type="cellIs" dxfId="5" priority="1771" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
+  <conditionalFormatting sqref="F365">
     <cfRule type="cellIs" dxfId="4" priority="1772" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
+  <conditionalFormatting sqref="F365">
     <cfRule type="cellIs" dxfId="5" priority="1773" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
+  <conditionalFormatting sqref="F365">
     <cfRule type="cellIs" dxfId="4" priority="1774" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
+  <conditionalFormatting sqref="F365">
     <cfRule type="cellIs" dxfId="5" priority="1775" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1776" operator="greaterThanOrEqual">
+  <conditionalFormatting sqref="E365">
+    <cfRule type="cellIs" dxfId="6" priority="1776" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18496,8 +18496,8 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1778" operator="lessThan">
-      <formula>-4100</formula>
+    <cfRule type="cellIs" dxfId="4" priority="1778" operator="greaterThanOrEqual">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F229">
@@ -18506,71 +18506,71 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1780" operator="greaterThanOrEqual">
-      <formula>0</formula>
+    <cfRule type="cellIs" dxfId="5" priority="1780" operator="lessThan">
+      <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1781" operator="lessThan">
-      <formula>-4100</formula>
+    <cfRule type="cellIs" dxfId="4" priority="1781" operator="greaterThanOrEqual">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1782" operator="greaterThanOrEqual">
-      <formula>0</formula>
+    <cfRule type="cellIs" dxfId="5" priority="1782" operator="lessThan">
+      <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1783" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="1783" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1784" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1785" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1786" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1787" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1788" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1789" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1790" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1791" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1792" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E229">
-    <cfRule type="cellIs" dxfId="6" priority="1784" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="5" priority="1785" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="4" priority="1786" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="4" priority="1787" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="5" priority="1788" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="4" priority="1789" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="5" priority="1790" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="4" priority="1791" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="5" priority="1792" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E365">
     <cfRule type="cellIs" dxfId="6" priority="1793" operator="greaterThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
📄 Replace ledger with Chuck's 10:07 upload: 84 open pairs (+1 new 09-24 763/2382 @22.38/65.4, 19 stored P/L refined)
</commit_message>
<xml_diff>
--- a/data/Record_Sept-24.xlsx
+++ b/data/Record_Sept-24.xlsx
@@ -1977,10 +1977,10 @@
       </c>
       <c r="H70" s="5" t="str">
         <f t="shared" ref="H70:H71" si="6">(I70-K70)/K70-$D$3</f>
-        <v>-1.98%</v>
+        <v>-2.40%</v>
       </c>
       <c r="I70" s="9">
-        <v>22.48</v>
+        <v>22.38</v>
       </c>
       <c r="J70" s="10">
         <v>763.0</v>
@@ -1998,10 +1998,10 @@
       </c>
       <c r="H71" s="5" t="str">
         <f t="shared" si="6"/>
-        <v>-5.03%</v>
+        <v>-4.61%</v>
       </c>
       <c r="I71" s="11">
-        <v>65.1</v>
+        <v>65.4</v>
       </c>
       <c r="J71" s="12">
         <v>2382.0</v>
@@ -2020,17 +2020,17 @@
       </c>
       <c r="H72" s="5" t="str">
         <f>H70-H71</f>
-        <v>3.05%</v>
+        <v>2.21%</v>
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="15" t="str">
         <f>I70</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B73" s="15" t="str">
         <f>I71</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C73">
         <v>600.0</v>
@@ -2094,11 +2094,11 @@
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B78" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="C78" s="16">
         <v>300.0</v>
@@ -2111,11 +2111,11 @@
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="4" t="str">
         <f>(A78-A77)*C78</f>
-        <v>-3600</v>
+        <v>-3510</v>
       </c>
       <c r="B79" s="14" t="str">
         <f>C79*(B77-B78)</f>
-        <v> $ 2,080.00 </v>
+        <v> $ 2,180.00 </v>
       </c>
       <c r="C79" s="16">
         <v>1000.0</v>
@@ -2125,11 +2125,11 @@
       </c>
       <c r="E79" s="14" t="str">
         <f>A79</f>
-        <v>-$ 3,600.00 </v>
+        <v>-$ 3,510.00 </v>
       </c>
       <c r="F79" s="14" t="str">
         <f>(B79+A79)</f>
-        <v>-$ 1,520.00 </v>
+        <v>-$ 1,330.00 </v>
       </c>
       <c r="G79" t="str">
         <f>IF(F79&gt;0, "TRADE","H")</f>
@@ -2169,11 +2169,11 @@
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B83" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="C83">
         <v>200.0</v>
@@ -2186,11 +2186,11 @@
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="4" t="str">
         <f>(A83-A82)*C83</f>
-        <v>-2180</v>
+        <v>-2120</v>
       </c>
       <c r="B84" s="14" t="str">
         <f>C84*(B82-B83)</f>
-        <v> $ 1,308.00 </v>
+        <v> $ 1,368.00 </v>
       </c>
       <c r="C84">
         <v>600.0</v>
@@ -2200,11 +2200,11 @@
       </c>
       <c r="E84" s="14" t="str">
         <f>A84</f>
-        <v>-$ 2,180.00 </v>
+        <v>-$ 2,120.00 </v>
       </c>
       <c r="F84" s="14" t="str">
         <f>(B84+A84)</f>
-        <v>-$ 872.00 </v>
+        <v>-$ 752.00 </v>
       </c>
       <c r="G84" t="str">
         <f>IF(F84&gt;0, "TRADE","H")</f>
@@ -2244,11 +2244,11 @@
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B88" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="C88">
         <v>200.0</v>
@@ -2261,11 +2261,11 @@
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="4" t="str">
         <f>(A88-A87)*C88</f>
-        <v>-510</v>
+        <v>-450</v>
       </c>
       <c r="B89" s="14" t="str">
         <f>C89*(B87-B88)</f>
-        <v> $ 180.00 </v>
+        <v> $ 240.00 </v>
       </c>
       <c r="C89">
         <v>600.0</v>
@@ -2275,11 +2275,11 @@
       </c>
       <c r="E89" s="14" t="str">
         <f>A89</f>
-        <v>-$ 510.00 </v>
+        <v>-$ 450.00 </v>
       </c>
       <c r="F89" s="14" t="str">
         <f>(B89+A89)</f>
-        <v>-$ 330.00 </v>
+        <v>-$ 210.00 </v>
       </c>
       <c r="G89" t="str">
         <f>IF(F89&gt;0, "TRADE","H")</f>
@@ -2319,11 +2319,11 @@
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B93" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="C93">
         <v>200.0</v>
@@ -2336,11 +2336,11 @@
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="4" t="str">
         <f>(A93-A92)*C93</f>
-        <v>-400</v>
+        <v>-340</v>
       </c>
       <c r="B94" s="14" t="str">
         <f>C94*(B92-B93)</f>
-        <v> $ 264.00 </v>
+        <v> $ 324.00 </v>
       </c>
       <c r="C94">
         <v>600.0</v>
@@ -2350,11 +2350,11 @@
       </c>
       <c r="E94" s="14" t="str">
         <f>A94</f>
-        <v>-$ 400.00 </v>
+        <v>-$ 340.00 </v>
       </c>
       <c r="F94" s="14" t="str">
         <f>(B94+A94)</f>
-        <v>-$ 136.00 </v>
+        <v>-$ 16.00 </v>
       </c>
       <c r="G94" t="str">
         <f>IF(F94&gt;0, "TRADE","H")</f>
@@ -2370,38 +2370,37 @@
         <v>6</v>
       </c>
       <c r="C95" s="8">
-        <v>46288.0</v>
+        <v>46289.0</v>
       </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="4">
+        <v>763.0</v>
+      </c>
+      <c r="B96" s="4">
         <v>2382.0</v>
       </c>
-      <c r="B96" s="4">
-        <v>763.0</v>
-      </c>
-      <c r="I96" s="17"/>
       <c r="M96" s="6"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="13">
-        <v>65.9</v>
+        <v>22.38</v>
       </c>
       <c r="B97" s="14">
-        <v>22.94</v>
+        <v>65.4</v>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="14" t="str">
+        <f>$A$73</f>
+        <v> $ 22.38 </v>
+      </c>
+      <c r="B98" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
-      </c>
-      <c r="B98" s="14" t="str">
-        <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C98">
-        <v>200.0</v>
+        <v>600.0</v>
       </c>
       <c r="D98" t="s">
         <v>8</v>
@@ -2411,29 +2410,29 @@
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="4" t="str">
         <f>(A98-A97)*C98</f>
-        <v>-160</v>
+        <v>0</v>
       </c>
       <c r="B99" s="14" t="str">
         <f>C99*(B97-B98)</f>
-        <v> $ 276.00 </v>
+        <v> $ -   </v>
       </c>
       <c r="C99">
-        <v>600.0</v>
+        <v>200.0</v>
       </c>
       <c r="D99" t="s">
         <v>9</v>
       </c>
       <c r="E99" s="14" t="str">
         <f>A99</f>
-        <v>-$ 160.00 </v>
+        <v> $ -   </v>
       </c>
       <c r="F99" s="14" t="str">
         <f>(B99+A99)</f>
-        <v> $ 116.00 </v>
+        <v> $ -   </v>
       </c>
       <c r="G99" t="str">
         <f>IF(F99&gt;0, "TRADE","H")</f>
-        <v>TRADE</v>
+        <v>H</v>
       </c>
       <c r="V99" s="6"/>
     </row>
@@ -2468,11 +2467,11 @@
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B103" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C103">
         <v>600.0</v>
@@ -2485,11 +2484,11 @@
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="4" t="str">
         <f>(A103-A102)*C103</f>
-        <v>-768</v>
+        <v>-828</v>
       </c>
       <c r="B104" s="14" t="str">
         <f>C104*(B102-B103)</f>
-        <v> $ 170.00 </v>
+        <v> $ 110.00 </v>
       </c>
       <c r="C104">
         <v>200.0</v>
@@ -2499,11 +2498,11 @@
       </c>
       <c r="E104" s="14" t="str">
         <f>A104</f>
-        <v>-$ 768.00 </v>
+        <v>-$ 828.00 </v>
       </c>
       <c r="F104" s="14" t="str">
         <f>(B104+A104)</f>
-        <v>-$ 598.00 </v>
+        <v>-$ 718.00 </v>
       </c>
       <c r="G104" t="str">
         <f>IF(F104&gt;0, "TRADE","H")</f>
@@ -2542,11 +2541,11 @@
     <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B108" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C108">
         <v>600.0</v>
@@ -2559,11 +2558,11 @@
     <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="4" t="str">
         <f>(A108-A107)*C108</f>
-        <v>-504</v>
+        <v>-564</v>
       </c>
       <c r="B109" s="14" t="str">
         <f>C109*(B107-B108)</f>
-        <v>-$ 890.00 </v>
+        <v>-$ 950.00 </v>
       </c>
       <c r="C109">
         <v>200.0</v>
@@ -2573,11 +2572,11 @@
       </c>
       <c r="E109" s="14" t="str">
         <f>A109</f>
-        <v>-$ 504.00 </v>
+        <v>-$ 564.00 </v>
       </c>
       <c r="F109" s="14" t="str">
         <f>(B109+A109)</f>
-        <v>-$ 1,394.00 </v>
+        <v>-$ 1,514.00 </v>
       </c>
       <c r="G109" t="str">
         <f>IF(F109&gt;0, "TRADE","H")</f>
@@ -2616,11 +2615,11 @@
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B113" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C113">
         <v>600.0</v>
@@ -2633,11 +2632,11 @@
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="4" t="str">
         <f>(A113-A112)*C113</f>
-        <v>-852</v>
+        <v>-912</v>
       </c>
       <c r="B114" s="14" t="str">
         <f>C114*(B112-B113)</f>
-        <v>-$ 1,070.00 </v>
+        <v>-$ 1,130.00 </v>
       </c>
       <c r="C114">
         <v>200.0</v>
@@ -2647,11 +2646,11 @@
       </c>
       <c r="E114" s="14" t="str">
         <f>A114</f>
-        <v>-$ 852.00 </v>
+        <v>-$ 912.00 </v>
       </c>
       <c r="F114" s="14" t="str">
         <f>(B114+A114)</f>
-        <v>-$ 1,922.00 </v>
+        <v>-$ 2,042.00 </v>
       </c>
       <c r="G114" t="str">
         <f>IF(F114&gt;0, "TRADE","H")</f>
@@ -2690,11 +2689,11 @@
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B118" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C118">
         <v>600.0</v>
@@ -2707,11 +2706,11 @@
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="4" t="str">
         <f>(A118-A117)*C118</f>
-        <v>-1824</v>
+        <v>-1884</v>
       </c>
       <c r="B119" s="14" t="str">
         <f>C119*(B117-B118)</f>
-        <v>-$ 560.00 </v>
+        <v>-$ 620.00 </v>
       </c>
       <c r="C119">
         <v>200.0</v>
@@ -2721,11 +2720,11 @@
       </c>
       <c r="E119" s="14" t="str">
         <f>A119</f>
-        <v>-$ 1,824.00 </v>
+        <v>-$ 1,884.00 </v>
       </c>
       <c r="F119" s="14" t="str">
         <f>(B119+A119)</f>
-        <v>-$ 2,384.00 </v>
+        <v>-$ 2,504.00 </v>
       </c>
       <c r="G119" t="str">
         <f>IF(F119&gt;0, "TRADE","H")</f>
@@ -2764,11 +2763,11 @@
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B123" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C123">
         <v>600.0</v>
@@ -2781,11 +2780,11 @@
     <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="4" t="str">
         <f>(A123-A122)*C123</f>
-        <v>-1788</v>
+        <v>-1848</v>
       </c>
       <c r="B124" s="14" t="str">
         <f>C124*(B122-B123)</f>
-        <v>-$ 890.00 </v>
+        <v>-$ 950.00 </v>
       </c>
       <c r="C124">
         <v>200.0</v>
@@ -2795,11 +2794,11 @@
       </c>
       <c r="E124" s="14" t="str">
         <f>A124</f>
-        <v>-$ 1,788.00 </v>
+        <v>-$ 1,848.00 </v>
       </c>
       <c r="F124" s="14" t="str">
         <f>(B124+A124)</f>
-        <v>-$ 2,678.00 </v>
+        <v>-$ 2,798.00 </v>
       </c>
       <c r="G124" t="str">
         <f>IF(F124&gt;0, "TRADE","H")</f>
@@ -2838,11 +2837,11 @@
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B128" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C128">
         <v>600.0</v>
@@ -2855,11 +2854,11 @@
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="4" t="str">
         <f>(A128-A127)*C128</f>
-        <v>-1836</v>
+        <v>-1896</v>
       </c>
       <c r="B129" s="14" t="str">
         <f>C129*(B127-B128)</f>
-        <v>-$ 1,260.00 </v>
+        <v>-$ 1,320.00 </v>
       </c>
       <c r="C129">
         <v>200.0</v>
@@ -2869,11 +2868,11 @@
       </c>
       <c r="E129" s="14" t="str">
         <f>A129</f>
-        <v>-$ 1,836.00 </v>
+        <v>-$ 1,896.00 </v>
       </c>
       <c r="F129" s="14" t="str">
         <f>(B129+A129)</f>
-        <v>-$ 3,096.00 </v>
+        <v>-$ 3,216.00 </v>
       </c>
       <c r="G129" t="str">
         <f>IF(F129&gt;0, "TRADE","H")</f>
@@ -2912,11 +2911,11 @@
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B133" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C133">
         <v>600.0</v>
@@ -2929,11 +2928,11 @@
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="4" t="str">
         <f>(A133-A132)*C133</f>
-        <v>-1824</v>
+        <v>-1884</v>
       </c>
       <c r="B134" s="14" t="str">
         <f>C134*(B132-B133)</f>
-        <v>-$ 1,720.00 </v>
+        <v>-$ 1,780.00 </v>
       </c>
       <c r="C134">
         <v>200.0</v>
@@ -2943,11 +2942,11 @@
       </c>
       <c r="E134" s="14" t="str">
         <f>A134</f>
-        <v>-$ 1,824.00 </v>
+        <v>-$ 1,884.00 </v>
       </c>
       <c r="F134" s="14" t="str">
         <f>(B134+A134)</f>
-        <v>-$ 3,544.00 </v>
+        <v>-$ 3,664.00 </v>
       </c>
       <c r="G134" t="str">
         <f>IF(F134&gt;0, "TRADE","H")</f>
@@ -2986,11 +2985,11 @@
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B138" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C138">
         <v>600.0</v>
@@ -3003,11 +3002,11 @@
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="4" t="str">
         <f>(A138-A137)*C138</f>
-        <v>-2016</v>
+        <v>-2076</v>
       </c>
       <c r="B139" s="14" t="str">
         <f>C139*(B137-B138)</f>
-        <v>-$ 1,670.00 </v>
+        <v>-$ 1,730.00 </v>
       </c>
       <c r="C139">
         <v>200.0</v>
@@ -3017,11 +3016,11 @@
       </c>
       <c r="E139" s="14" t="str">
         <f>A139</f>
-        <v>-$ 2,016.00 </v>
+        <v>-$ 2,076.00 </v>
       </c>
       <c r="F139" s="14" t="str">
         <f>(B139+A139)</f>
-        <v>-$ 3,686.00 </v>
+        <v>-$ 3,806.00 </v>
       </c>
       <c r="G139" t="str">
         <f>IF(F139&gt;0, "TRADE","H")</f>
@@ -3062,11 +3061,11 @@
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="14" t="str">
         <f>$A$73</f>
-        <v> $ 22.48 </v>
+        <v> $ 22.38 </v>
       </c>
       <c r="B143" s="14" t="str">
         <f>$B$73</f>
-        <v> $ 65.10 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C143">
         <v>600.0</v>
@@ -3079,11 +3078,11 @@
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="4" t="str">
         <f>(A143-A142)*C143</f>
-        <v>-4482</v>
+        <v>-4542</v>
       </c>
       <c r="B144" s="14" t="str">
         <f>C144*(B142-B143)</f>
-        <v>-$ 49.20 </v>
+        <v>-$ 109.20 </v>
       </c>
       <c r="C144">
         <v>200.0</v>
@@ -3093,11 +3092,11 @@
       </c>
       <c r="E144" s="14" t="str">
         <f>A144</f>
-        <v>-$ 4,482.00 </v>
+        <v>-$ 4,542.00 </v>
       </c>
       <c r="F144" s="14" t="str">
         <f>(B144+A144)</f>
-        <v>-$ 4,531.20 </v>
+        <v>-$ 4,651.20 </v>
       </c>
       <c r="G144" t="str">
         <f>IF(F144&gt;0, "TRADE","H")</f>
@@ -5453,10 +5452,10 @@
       </c>
       <c r="H276" s="5" t="str">
         <f t="shared" ref="H276:H277" si="14">(I276-K276)/K276-$D$3</f>
-        <v>-4.82%</v>
+        <v>-4.61%</v>
       </c>
       <c r="I276" s="9">
-        <v>65.25</v>
+        <v>65.4</v>
       </c>
       <c r="J276" s="10">
         <v>2382.0</v>
@@ -5475,10 +5474,10 @@
       </c>
       <c r="H277" s="5" t="str">
         <f t="shared" si="14"/>
-        <v>-6.21%</v>
+        <v>-5.95%</v>
       </c>
       <c r="I277" s="9">
-        <v>86.95</v>
+        <v>87.2</v>
       </c>
       <c r="J277" s="12" t="s">
         <v>10</v>
@@ -5496,7 +5495,7 @@
       </c>
       <c r="H278" s="5" t="str">
         <f>H276-H277</f>
-        <v>1.39%</v>
+        <v>1.34%</v>
       </c>
       <c r="I278" s="17"/>
       <c r="Y278" s="6"/>
@@ -5504,11 +5503,11 @@
     <row r="279" ht="15.75" customHeight="1">
       <c r="A279" s="15" t="str">
         <f>I276</f>
-        <v> $ 65.25 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B279" s="15" t="str">
         <f>I277</f>
-        <v> $ 86.95 </v>
+        <v> $ 87.20 </v>
       </c>
       <c r="C279">
         <v>200.0</v>
@@ -5570,11 +5569,11 @@
     <row r="284" ht="15.75" customHeight="1">
       <c r="A284" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 86.95 </v>
+        <v> $ 87.20 </v>
       </c>
       <c r="B284" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 65.25 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="C284">
         <v>200.0</v>
@@ -5585,22 +5584,22 @@
     <row r="285" ht="15.75" customHeight="1">
       <c r="A285" s="4" t="str">
         <f>(A284-A283)*C285</f>
-        <v>-1350</v>
+        <v>-1300</v>
       </c>
       <c r="B285" s="4" t="str">
         <f>(B283-B284)*C284</f>
-        <v>550</v>
+        <v>520</v>
       </c>
       <c r="C285">
         <v>200.0</v>
       </c>
       <c r="E285" s="14" t="str">
         <f>A285</f>
-        <v>-$ 1,350.00 </v>
+        <v>-$ 1,300.00 </v>
       </c>
       <c r="F285" s="4" t="str">
         <f>(B285+A285)</f>
-        <v>-800</v>
+        <v>-780</v>
       </c>
       <c r="G285" t="str">
         <f>IF(F285&gt;0, "TRADE","H")</f>
@@ -5645,11 +5644,11 @@
     <row r="289" ht="15.75" customHeight="1">
       <c r="A289" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 65.25 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B289" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 86.95 </v>
+        <v> $ 87.20 </v>
       </c>
       <c r="C289">
         <v>200.0</v>
@@ -5660,22 +5659,22 @@
     <row r="290" ht="15.75" customHeight="1">
       <c r="A290" s="4" t="str">
         <f>(A289-A288)*C290</f>
-        <v>-350</v>
+        <v>-320</v>
       </c>
       <c r="B290" s="4" t="str">
         <f>(B288-B289)*C289</f>
-        <v>510</v>
+        <v>460</v>
       </c>
       <c r="C290">
         <v>200.0</v>
       </c>
       <c r="E290" s="14" t="str">
         <f>A290</f>
-        <v>-$ 350.00 </v>
+        <v>-$ 320.00 </v>
       </c>
       <c r="F290" s="4" t="str">
         <f>(B290+A290)</f>
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="G290" t="str">
         <f>IF(F290&gt;0, "TRADE","H")</f>
@@ -5721,11 +5720,11 @@
     <row r="294" ht="15.75" customHeight="1">
       <c r="A294" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 65.25 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B294" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 86.95 </v>
+        <v> $ 87.20 </v>
       </c>
       <c r="C294">
         <v>200.0</v>
@@ -5736,22 +5735,22 @@
     <row r="295" ht="15.75" customHeight="1">
       <c r="A295" s="4" t="str">
         <f>(A294-A293)*C295</f>
-        <v>-3438.8</v>
+        <v>-3408.8</v>
       </c>
       <c r="B295" s="4" t="str">
         <f>(B293-B294)*C294</f>
-        <v>1390</v>
+        <v>1340</v>
       </c>
       <c r="C295">
         <v>200.0</v>
       </c>
       <c r="E295" s="14" t="str">
         <f>A295</f>
-        <v>-$ 3,438.80 </v>
+        <v>-$ 3,408.80 </v>
       </c>
       <c r="F295" s="4" t="str">
         <f>(B295+A295)</f>
-        <v>-2048.8</v>
+        <v>-2068.8</v>
       </c>
       <c r="G295" t="str">
         <f>IF(F295&gt;0, "TRADE","H")</f>
@@ -5797,11 +5796,11 @@
     <row r="299" ht="15.75" customHeight="1">
       <c r="A299" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 65.25 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B299" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 86.95 </v>
+        <v> $ 87.20 </v>
       </c>
       <c r="C299">
         <v>200.0</v>
@@ -5812,22 +5811,22 @@
     <row r="300" ht="15.75" customHeight="1">
       <c r="A300" s="4" t="str">
         <f>(A299-A298)*C300</f>
-        <v>-3418.8</v>
+        <v>-3388.8</v>
       </c>
       <c r="B300" s="4" t="str">
         <f>(B298-B299)*C299</f>
-        <v>550</v>
+        <v>500</v>
       </c>
       <c r="C300">
         <v>200.0</v>
       </c>
       <c r="E300" s="14" t="str">
         <f>A300</f>
-        <v>-$ 3,418.80 </v>
+        <v>-$ 3,388.80 </v>
       </c>
       <c r="F300" s="4" t="str">
         <f>(B300+A300)</f>
-        <v>-2868.8</v>
+        <v>-2888.8</v>
       </c>
       <c r="G300" t="str">
         <f>IF(F300&gt;0, "TRADE","H")</f>
@@ -5873,11 +5872,11 @@
     <row r="304" ht="15.75" customHeight="1">
       <c r="A304" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 65.25 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B304" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 86.95 </v>
+        <v> $ 87.20 </v>
       </c>
       <c r="C304">
         <v>200.0</v>
@@ -5888,22 +5887,22 @@
     <row r="305" ht="15.75" customHeight="1">
       <c r="A305" s="4" t="str">
         <f>(A304-A303)*C305</f>
-        <v>-3108.8</v>
+        <v>-3078.8</v>
       </c>
       <c r="B305" s="4" t="str">
         <f>(B303-B304)*C304</f>
-        <v>190</v>
+        <v>140</v>
       </c>
       <c r="C305">
         <v>200.0</v>
       </c>
       <c r="E305" s="14" t="str">
         <f>A305</f>
-        <v>-$ 3,108.80 </v>
+        <v>-$ 3,078.80 </v>
       </c>
       <c r="F305" s="4" t="str">
         <f>(B305+A305)</f>
-        <v>-2918.8</v>
+        <v>-2938.8</v>
       </c>
       <c r="G305" t="str">
         <f>IF(F305&gt;0, "TRADE","H")</f>
@@ -5949,11 +5948,11 @@
     <row r="309" ht="15.75" customHeight="1">
       <c r="A309" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 65.25 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B309" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 86.95 </v>
+        <v> $ 87.20 </v>
       </c>
       <c r="C309">
         <v>200.0</v>
@@ -5964,22 +5963,22 @@
     <row r="310" ht="15.75" customHeight="1">
       <c r="A310" s="4" t="str">
         <f>(A309-A308)*C310</f>
-        <v>-3452.4</v>
+        <v>-3422.4</v>
       </c>
       <c r="B310" s="4" t="str">
         <f>(B308-B309)*C309</f>
-        <v>-610</v>
+        <v>-660</v>
       </c>
       <c r="C310">
         <v>200.0</v>
       </c>
       <c r="E310" s="14" t="str">
         <f>A310</f>
-        <v>-$ 3,452.40 </v>
+        <v>-$ 3,422.40 </v>
       </c>
       <c r="F310" s="4" t="str">
         <f>(B310+A310)</f>
-        <v>-4062.4</v>
+        <v>-4082.4</v>
       </c>
       <c r="G310" t="str">
         <f>IF(F310&gt;0, "TRADE","H")</f>
@@ -6025,11 +6024,11 @@
     <row r="314" ht="15.75" customHeight="1">
       <c r="A314" s="14" t="str">
         <f>$A$279</f>
-        <v> $ 65.25 </v>
+        <v> $ 65.40 </v>
       </c>
       <c r="B314" s="14" t="str">
         <f>$B$279</f>
-        <v> $ 86.95 </v>
+        <v> $ 87.20 </v>
       </c>
       <c r="C314">
         <v>200.0</v>
@@ -6040,22 +6039,22 @@
     <row r="315" ht="15.75" customHeight="1">
       <c r="A315" s="4" t="str">
         <f>(A314-A313)*C315</f>
-        <v>-3452.4</v>
+        <v>-3422.4</v>
       </c>
       <c r="B315" s="4" t="str">
         <f>(B313-B314)*C314</f>
-        <v>-610</v>
+        <v>-660</v>
       </c>
       <c r="C315">
         <v>200.0</v>
       </c>
       <c r="E315" s="14" t="str">
         <f>A315</f>
-        <v>-$ 3,452.40 </v>
+        <v>-$ 3,422.40 </v>
       </c>
       <c r="F315" s="4" t="str">
         <f>(B315+A315)</f>
-        <v>-4062.4</v>
+        <v>-4082.4</v>
       </c>
       <c r="G315" t="str">
         <f>IF(F315&gt;0, "TRADE","H")</f>
@@ -18360,217 +18359,217 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F365">
+    <cfRule type="cellIs" dxfId="5" priority="1751" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F365">
+    <cfRule type="cellIs" dxfId="4" priority="1752" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F365">
+    <cfRule type="cellIs" dxfId="4" priority="1753" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F365">
+    <cfRule type="cellIs" dxfId="5" priority="1754" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F365">
+    <cfRule type="cellIs" dxfId="4" priority="1755" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F365">
+    <cfRule type="cellIs" dxfId="5" priority="1756" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F365">
+    <cfRule type="cellIs" dxfId="4" priority="1757" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F365">
+    <cfRule type="cellIs" dxfId="5" priority="1758" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E365">
+    <cfRule type="cellIs" dxfId="6" priority="1759" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1760" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1761" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1762" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1763" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1764" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1765" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1766" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1767" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1768" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1769" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1770" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1771" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1772" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1773" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="4" priority="1774" operator="greaterThanOrEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F229">
+    <cfRule type="cellIs" dxfId="5" priority="1775" operator="lessThan">
+      <formula>-4100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E229">
+    <cfRule type="cellIs" dxfId="6" priority="1776" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="5" priority="1751" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="1777" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="4" priority="1752" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1778" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="4" priority="1753" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1779" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="5" priority="1754" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="1780" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="4" priority="1755" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1781" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="5" priority="1756" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="1782" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="4" priority="1757" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1783" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="5" priority="1758" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="1784" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="4" priority="1759" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1785" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="5" priority="1760" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="1786" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="5" priority="1761" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="1787" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="4" priority="1762" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1788" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="4" priority="1763" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1789" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="5" priority="1764" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="1790" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="4" priority="1765" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1791" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99">
-    <cfRule type="cellIs" dxfId="5" priority="1766" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="1792" operator="lessThan">
       <formula>-4100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E99">
-    <cfRule type="cellIs" dxfId="6" priority="1767" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="5" priority="1768" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="4" priority="1769" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="4" priority="1770" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="5" priority="1771" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="4" priority="1772" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="5" priority="1773" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="4" priority="1774" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F365">
-    <cfRule type="cellIs" dxfId="5" priority="1775" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E365">
-    <cfRule type="cellIs" dxfId="6" priority="1776" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1777" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1778" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1779" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1780" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1781" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1782" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1783" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1784" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1785" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1786" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1787" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1788" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1789" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1790" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="4" priority="1791" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F229">
-    <cfRule type="cellIs" dxfId="5" priority="1792" operator="lessThan">
-      <formula>-4100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E229">
     <cfRule type="cellIs" dxfId="6" priority="1793" operator="greaterThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>